<commit_message>
Add file upload + /export for two-way Excel sync
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline.xlsx
+++ b/pipeline.xlsx
@@ -570,7 +570,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -760,7 +759,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -844,7 +842,6 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1004,7 +1001,6 @@
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -2057,16 +2053,30 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n"/>
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Vikas Sharma</t>
+        </is>
+      </c>
       <c r="B12" s="12" t="n"/>
       <c r="C12" s="12" t="n"/>
       <c r="D12" s="12" t="n"/>
       <c r="E12" s="12" t="n"/>
-      <c r="F12" s="12" t="n"/>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
       <c r="G12" s="12" t="n"/>
-      <c r="H12" s="16" t="n"/>
+      <c r="H12" s="16" t="n">
+        <v>250000</v>
+      </c>
       <c r="I12" s="16" t="n"/>
-      <c r="J12" s="12" t="n"/>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K12" s="12" t="n"/>
       <c r="L12" s="17">
         <f>IF(A12="","",DAYS(TODAY(),J12))</f>
@@ -4854,10 +4864,12 @@
           <t>Active Deals</t>
         </is>
       </c>
+      <c r="B4" s="34" t="n"/>
       <c r="C4" s="37">
         <f>COUNTIFS(Pipeline!A5:A80,"&lt;&gt;",Pipeline!F5:F80,"&lt;&gt;Closed-Won",Pipeline!F5:F80,"&lt;&gt;Closed-Lost")</f>
         <v/>
       </c>
+      <c r="D4" s="34" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="36" t="inlineStr">
@@ -4865,10 +4877,12 @@
           <t>Pipeline Value</t>
         </is>
       </c>
+      <c r="B5" s="34" t="n"/>
       <c r="C5" s="38">
         <f>SUMPRODUCT((Pipeline!F5:F80&lt;&gt;"Closed-Won")*(Pipeline!F5:F80&lt;&gt;"Closed-Lost")*(Pipeline!F5:F80&lt;&gt;"")*Pipeline!H5:H80)</f>
         <v/>
       </c>
+      <c r="D5" s="34" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="36" t="inlineStr">
@@ -4876,10 +4890,12 @@
           <t>Hot Leads</t>
         </is>
       </c>
+      <c r="B6" s="34" t="n"/>
       <c r="C6" s="37">
         <f>COUNTIF(Pipeline!E5:E80,"Hot")</f>
         <v/>
       </c>
+      <c r="D6" s="34" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="36" t="inlineStr">
@@ -4887,10 +4903,12 @@
           <t>Overdue Follow-Ups</t>
         </is>
       </c>
+      <c r="B7" s="34" t="n"/>
       <c r="C7" s="37">
         <f>COUNTIFS(Pipeline!K5:K80,"&lt;"&amp;TODAY(),Pipeline!K5:K80,"&lt;&gt;",Pipeline!F5:F80,"&lt;&gt;Closed-Won",Pipeline!F5:F80,"&lt;&gt;Closed-Lost")</f>
         <v/>
       </c>
+      <c r="D7" s="34" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="36" t="inlineStr">
@@ -4898,10 +4916,12 @@
           <t>Follow-Ups This Week</t>
         </is>
       </c>
+      <c r="B8" s="34" t="n"/>
       <c r="C8" s="37">
         <f>COUNTIFS(Pipeline!K5:K80,"&gt;="&amp;TODAY(),Pipeline!K5:K80,"&lt;="&amp;(TODAY()+7),Pipeline!F5:F80,"&lt;&gt;Closed-Won")</f>
         <v/>
       </c>
+      <c r="D8" s="34" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="36" t="inlineStr">
@@ -4909,10 +4929,12 @@
           <t>Deals Won (Total)</t>
         </is>
       </c>
+      <c r="B9" s="34" t="n"/>
       <c r="C9" s="37">
         <f>COUNTIF(Pipeline!F5:F80,"Closed-Won")</f>
         <v/>
       </c>
+      <c r="D9" s="34" t="n"/>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="31" t="inlineStr">
@@ -4982,12 +5004,21 @@
     </row>
     <row r="20" ht="25" customHeight="1">
       <c r="A20" s="39" t="n"/>
+      <c r="B20" s="33" t="n"/>
+      <c r="C20" s="33" t="n"/>
+      <c r="D20" s="34" t="n"/>
     </row>
     <row r="21" ht="25" customHeight="1">
       <c r="A21" s="40" t="n"/>
+      <c r="B21" s="33" t="n"/>
+      <c r="C21" s="33" t="n"/>
+      <c r="D21" s="34" t="n"/>
     </row>
     <row r="22" ht="25" customHeight="1">
       <c r="A22" s="39" t="n"/>
+      <c r="B22" s="33" t="n"/>
+      <c r="C22" s="33" t="n"/>
+      <c r="D22" s="34" t="n"/>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="31" t="inlineStr">
@@ -5002,6 +5033,9 @@
           <t>1.</t>
         </is>
       </c>
+      <c r="B25" s="33" t="n"/>
+      <c r="C25" s="33" t="n"/>
+      <c r="D25" s="34" t="n"/>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="32" t="inlineStr">
@@ -5009,6 +5043,9 @@
           <t>2.</t>
         </is>
       </c>
+      <c r="B26" s="33" t="n"/>
+      <c r="C26" s="33" t="n"/>
+      <c r="D26" s="34" t="n"/>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="32" t="inlineStr">
@@ -5016,6 +5053,9 @@
           <t>3.</t>
         </is>
       </c>
+      <c r="B27" s="33" t="n"/>
+      <c r="C27" s="33" t="n"/>
+      <c r="D27" s="34" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="23">

</xml_diff>

<commit_message>
Wipe mock data - clean pipeline ready for real prospects
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline.xlsx
+++ b/pipeline.xlsx
@@ -252,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -275,36 +275,18 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -570,6 +552,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -759,6 +742,7 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -842,6 +826,7 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1001,6 +986,7 @@
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1463,7 +1449,7 @@
   <sheetPr>
     <tabColor rgb="001ABC9C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1623,466 +1609,148 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>Sarah Johnson</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>519-555-0101</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>sarah.j@email.com</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>Referral</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>Hot</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>Discovery Call</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>Life Insurance + Wealth</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="n">
-        <v>350000</v>
-      </c>
-      <c r="I5" s="9" t="n">
-        <v>4500</v>
-      </c>
-      <c r="J5" s="10" t="inlineStr">
-        <is>
-          <t>2026-02-15</t>
-        </is>
-      </c>
-      <c r="K5" s="10" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="L5" s="11">
+      <c r="A5" s="8" t="n"/>
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="8" t="n"/>
+      <c r="H5" s="9" t="n"/>
+      <c r="I5" s="9" t="n"/>
+      <c r="J5" s="8" t="n"/>
+      <c r="K5" s="8" t="n"/>
+      <c r="L5" s="10">
         <f>IF(A5="","",DAYS(TODAY(),J5))</f>
         <v/>
       </c>
-      <c r="M5" s="8" t="inlineStr">
-        <is>
-          <t>Couple, 2 kids. Needs term life + RRSP/TFSA strategy.</t>
-        </is>
-      </c>
+      <c r="M5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>David Chen</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>519-555-0202</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>d.chen@email.com</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>Warm</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>New Lead</t>
-        </is>
-      </c>
-      <c r="G6" s="12" t="inlineStr">
-        <is>
-          <t>Wealth Management</t>
-        </is>
-      </c>
-      <c r="H6" s="13" t="n">
-        <v>180000</v>
-      </c>
-      <c r="I6" s="13" t="n">
-        <v>1800</v>
-      </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>2026-03-10</t>
-        </is>
-      </c>
-      <c r="L6" s="15">
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="11" t="n"/>
+      <c r="G6" s="11" t="n"/>
+      <c r="H6" s="12" t="n"/>
+      <c r="I6" s="12" t="n"/>
+      <c r="J6" s="11" t="n"/>
+      <c r="K6" s="11" t="n"/>
+      <c r="L6" s="13">
         <f>IF(A6="","",DAYS(TODAY(),J6))</f>
         <v/>
       </c>
-      <c r="M6" s="12" t="inlineStr">
-        <is>
-          <t>Software dev. Downloaded retirement guide.</t>
-        </is>
-      </c>
+      <c r="M6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Jessica Williams</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>519-555-0303</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>jwilliams@email.com</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>Social Media</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>Hot</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Plan Presentation</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>Life Insurance + Wealth</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="n">
-        <v>420000</v>
-      </c>
-      <c r="I7" s="9" t="n">
-        <v>5200</v>
-      </c>
-      <c r="J7" s="10" t="inlineStr">
-        <is>
-          <t>2026-01-20</t>
-        </is>
-      </c>
-      <c r="K7" s="10" t="inlineStr">
-        <is>
-          <t>2026-03-14</t>
-        </is>
-      </c>
-      <c r="L7" s="11">
+      <c r="A7" s="8" t="n"/>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="8" t="n"/>
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="9" t="n"/>
+      <c r="J7" s="8" t="n"/>
+      <c r="K7" s="8" t="n"/>
+      <c r="L7" s="10">
         <f>IF(A7="","",DAYS(TODAY(),J7))</f>
         <v/>
       </c>
-      <c r="M7" s="8" t="inlineStr">
-        <is>
-          <t>Dual income. RESP + retirement + $1M term life.</t>
-        </is>
-      </c>
+      <c r="M7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Michael Brown</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>519-555-0404</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>m.brown@email.com</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>Seminar</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>Warm</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>Proposal Sent</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>Wealth Management</t>
-        </is>
-      </c>
-      <c r="H8" s="13" t="n">
-        <v>275000</v>
-      </c>
-      <c r="I8" s="13" t="n">
-        <v>2750</v>
-      </c>
-      <c r="J8" s="14" t="inlineStr">
-        <is>
-          <t>2026-02-01</t>
-        </is>
-      </c>
-      <c r="K8" s="14" t="inlineStr">
-        <is>
-          <t>2026-03-09</t>
-        </is>
-      </c>
-      <c r="L8" s="15">
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="11" t="n"/>
+      <c r="K8" s="11" t="n"/>
+      <c r="L8" s="13">
         <f>IF(A8="","",DAYS(TODAY(),J8))</f>
         <v/>
       </c>
-      <c r="M8" s="12" t="inlineStr">
-        <is>
-          <t>Business owner. Corp investing + personal.</t>
-        </is>
-      </c>
+      <c r="M8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Priya Patel</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>519-555-0808</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>p.patel@email.com</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Referral</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>Hot</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Negotiation</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Life Insurance + Wealth</t>
-        </is>
-      </c>
-      <c r="H9" s="9" t="n">
-        <v>850000</v>
-      </c>
-      <c r="I9" s="9" t="n">
-        <v>10500</v>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
-        <is>
-          <t>2026-01-15</t>
-        </is>
-      </c>
-      <c r="K9" s="10" t="inlineStr">
-        <is>
-          <t>2026-03-10</t>
-        </is>
-      </c>
-      <c r="L9" s="11">
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="8" t="n"/>
+      <c r="H9" s="9" t="n"/>
+      <c r="I9" s="9" t="n"/>
+      <c r="J9" s="8" t="n"/>
+      <c r="K9" s="8" t="n"/>
+      <c r="L9" s="10">
         <f>IF(A9="","",DAYS(TODAY(),J9))</f>
         <v/>
       </c>
-      <c r="M9" s="8" t="inlineStr">
-        <is>
-          <t>Physician. IPP, corp life, key person insurance.</t>
-        </is>
-      </c>
+      <c r="M9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Amanda Taylor</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>519-555-0505</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>ataylor@email.com</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>Referral</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>Hot</t>
-        </is>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
-        <is>
-          <t>Closed-Won</t>
-        </is>
-      </c>
-      <c r="G10" s="12" t="inlineStr">
-        <is>
-          <t>Wealth Management</t>
-        </is>
-      </c>
-      <c r="H10" s="13" t="n">
-        <v>500000</v>
-      </c>
-      <c r="I10" s="13" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J10" s="14" t="inlineStr">
-        <is>
-          <t>2025-12-10</t>
-        </is>
-      </c>
-      <c r="K10" s="14" t="inlineStr"/>
-      <c r="L10" s="15">
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="12" t="n"/>
+      <c r="I10" s="12" t="n"/>
+      <c r="J10" s="11" t="n"/>
+      <c r="K10" s="11" t="n"/>
+      <c r="L10" s="13">
         <f>IF(A10="","",DAYS(TODAY(),J10))</f>
         <v/>
       </c>
-      <c r="M10" s="12" t="inlineStr">
-        <is>
-          <t>Full plan + investment mgmt. Great referral source.</t>
-        </is>
-      </c>
+      <c r="M10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Tyler Brooks</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>519-555-0909</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>t.brooks@email.com</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Cold Outreach</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>Cold</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Nurture</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>Life Insurance</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="9" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J11" s="10" t="inlineStr">
-        <is>
-          <t>2026-01-05</t>
-        </is>
-      </c>
-      <c r="K11" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="L11" s="11">
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="9" t="n"/>
+      <c r="I11" s="9" t="n"/>
+      <c r="J11" s="8" t="n"/>
+      <c r="K11" s="8" t="n"/>
+      <c r="L11" s="10">
         <f>IF(A11="","",DAYS(TODAY(),J11))</f>
         <v/>
       </c>
-      <c r="M11" s="8" t="inlineStr">
-        <is>
-          <t>Young professional. Term life quote sent. Not ready for wealth.</t>
-        </is>
-      </c>
+      <c r="M11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>Vikas Sharma</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="12" t="n"/>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="12" t="n"/>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t>New Lead</t>
-        </is>
-      </c>
-      <c r="G12" s="12" t="n"/>
-      <c r="H12" s="16" t="n">
-        <v>250000</v>
-      </c>
-      <c r="I12" s="16" t="n"/>
-      <c r="J12" s="12" t="inlineStr">
-        <is>
-          <t>2026-03-09</t>
-        </is>
-      </c>
-      <c r="K12" s="12" t="n"/>
-      <c r="L12" s="17">
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="12" t="n"/>
+      <c r="I12" s="12" t="n"/>
+      <c r="J12" s="11" t="n"/>
+      <c r="K12" s="11" t="n"/>
+      <c r="L12" s="13">
         <f>IF(A12="","",DAYS(TODAY(),J12))</f>
         <v/>
       </c>
-      <c r="M12" s="12" t="n"/>
+      <c r="M12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n"/>
@@ -2092,33 +1760,33 @@
       <c r="E13" s="8" t="n"/>
       <c r="F13" s="8" t="n"/>
       <c r="G13" s="8" t="n"/>
-      <c r="H13" s="18" t="n"/>
-      <c r="I13" s="18" t="n"/>
+      <c r="H13" s="9" t="n"/>
+      <c r="I13" s="9" t="n"/>
       <c r="J13" s="8" t="n"/>
       <c r="K13" s="8" t="n"/>
-      <c r="L13" s="19">
+      <c r="L13" s="10">
         <f>IF(A13="","",DAYS(TODAY(),J13))</f>
         <v/>
       </c>
       <c r="M13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="12" t="n"/>
-      <c r="F14" s="12" t="n"/>
-      <c r="G14" s="12" t="n"/>
-      <c r="H14" s="16" t="n"/>
-      <c r="I14" s="16" t="n"/>
-      <c r="J14" s="12" t="n"/>
-      <c r="K14" s="12" t="n"/>
-      <c r="L14" s="17">
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
+      <c r="H14" s="12" t="n"/>
+      <c r="I14" s="12" t="n"/>
+      <c r="J14" s="11" t="n"/>
+      <c r="K14" s="11" t="n"/>
+      <c r="L14" s="13">
         <f>IF(A14="","",DAYS(TODAY(),J14))</f>
         <v/>
       </c>
-      <c r="M14" s="12" t="n"/>
+      <c r="M14" s="11" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n"/>
@@ -2128,33 +1796,33 @@
       <c r="E15" s="8" t="n"/>
       <c r="F15" s="8" t="n"/>
       <c r="G15" s="8" t="n"/>
-      <c r="H15" s="18" t="n"/>
-      <c r="I15" s="18" t="n"/>
+      <c r="H15" s="9" t="n"/>
+      <c r="I15" s="9" t="n"/>
       <c r="J15" s="8" t="n"/>
       <c r="K15" s="8" t="n"/>
-      <c r="L15" s="19">
+      <c r="L15" s="10">
         <f>IF(A15="","",DAYS(TODAY(),J15))</f>
         <v/>
       </c>
       <c r="M15" s="8" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="12" t="n"/>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="12" t="n"/>
-      <c r="F16" s="12" t="n"/>
-      <c r="G16" s="12" t="n"/>
-      <c r="H16" s="16" t="n"/>
-      <c r="I16" s="16" t="n"/>
-      <c r="J16" s="12" t="n"/>
-      <c r="K16" s="12" t="n"/>
-      <c r="L16" s="17">
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
+      <c r="H16" s="12" t="n"/>
+      <c r="I16" s="12" t="n"/>
+      <c r="J16" s="11" t="n"/>
+      <c r="K16" s="11" t="n"/>
+      <c r="L16" s="13">
         <f>IF(A16="","",DAYS(TODAY(),J16))</f>
         <v/>
       </c>
-      <c r="M16" s="12" t="n"/>
+      <c r="M16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n"/>
@@ -2164,33 +1832,33 @@
       <c r="E17" s="8" t="n"/>
       <c r="F17" s="8" t="n"/>
       <c r="G17" s="8" t="n"/>
-      <c r="H17" s="18" t="n"/>
-      <c r="I17" s="18" t="n"/>
+      <c r="H17" s="9" t="n"/>
+      <c r="I17" s="9" t="n"/>
       <c r="J17" s="8" t="n"/>
       <c r="K17" s="8" t="n"/>
-      <c r="L17" s="19">
+      <c r="L17" s="10">
         <f>IF(A17="","",DAYS(TODAY(),J17))</f>
         <v/>
       </c>
       <c r="M17" s="8" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="12" t="n"/>
-      <c r="E18" s="12" t="n"/>
-      <c r="F18" s="12" t="n"/>
-      <c r="G18" s="12" t="n"/>
-      <c r="H18" s="16" t="n"/>
-      <c r="I18" s="16" t="n"/>
-      <c r="J18" s="12" t="n"/>
-      <c r="K18" s="12" t="n"/>
-      <c r="L18" s="17">
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
+      <c r="H18" s="12" t="n"/>
+      <c r="I18" s="12" t="n"/>
+      <c r="J18" s="11" t="n"/>
+      <c r="K18" s="11" t="n"/>
+      <c r="L18" s="13">
         <f>IF(A18="","",DAYS(TODAY(),J18))</f>
         <v/>
       </c>
-      <c r="M18" s="12" t="n"/>
+      <c r="M18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n"/>
@@ -2200,33 +1868,33 @@
       <c r="E19" s="8" t="n"/>
       <c r="F19" s="8" t="n"/>
       <c r="G19" s="8" t="n"/>
-      <c r="H19" s="18" t="n"/>
-      <c r="I19" s="18" t="n"/>
+      <c r="H19" s="9" t="n"/>
+      <c r="I19" s="9" t="n"/>
       <c r="J19" s="8" t="n"/>
       <c r="K19" s="8" t="n"/>
-      <c r="L19" s="19">
+      <c r="L19" s="10">
         <f>IF(A19="","",DAYS(TODAY(),J19))</f>
         <v/>
       </c>
       <c r="M19" s="8" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="12" t="n"/>
-      <c r="F20" s="12" t="n"/>
-      <c r="G20" s="12" t="n"/>
-      <c r="H20" s="16" t="n"/>
-      <c r="I20" s="16" t="n"/>
-      <c r="J20" s="12" t="n"/>
-      <c r="K20" s="12" t="n"/>
-      <c r="L20" s="17">
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
+      <c r="G20" s="11" t="n"/>
+      <c r="H20" s="12" t="n"/>
+      <c r="I20" s="12" t="n"/>
+      <c r="J20" s="11" t="n"/>
+      <c r="K20" s="11" t="n"/>
+      <c r="L20" s="13">
         <f>IF(A20="","",DAYS(TODAY(),J20))</f>
         <v/>
       </c>
-      <c r="M20" s="12" t="n"/>
+      <c r="M20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n"/>
@@ -2236,33 +1904,33 @@
       <c r="E21" s="8" t="n"/>
       <c r="F21" s="8" t="n"/>
       <c r="G21" s="8" t="n"/>
-      <c r="H21" s="18" t="n"/>
-      <c r="I21" s="18" t="n"/>
+      <c r="H21" s="9" t="n"/>
+      <c r="I21" s="9" t="n"/>
       <c r="J21" s="8" t="n"/>
       <c r="K21" s="8" t="n"/>
-      <c r="L21" s="19">
+      <c r="L21" s="10">
         <f>IF(A21="","",DAYS(TODAY(),J21))</f>
         <v/>
       </c>
       <c r="M21" s="8" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="n"/>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="12" t="n"/>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="12" t="n"/>
-      <c r="F22" s="12" t="n"/>
-      <c r="G22" s="12" t="n"/>
-      <c r="H22" s="16" t="n"/>
-      <c r="I22" s="16" t="n"/>
-      <c r="J22" s="12" t="n"/>
-      <c r="K22" s="12" t="n"/>
-      <c r="L22" s="17">
+      <c r="A22" s="11" t="n"/>
+      <c r="B22" s="11" t="n"/>
+      <c r="C22" s="11" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="11" t="n"/>
+      <c r="G22" s="11" t="n"/>
+      <c r="H22" s="12" t="n"/>
+      <c r="I22" s="12" t="n"/>
+      <c r="J22" s="11" t="n"/>
+      <c r="K22" s="11" t="n"/>
+      <c r="L22" s="13">
         <f>IF(A22="","",DAYS(TODAY(),J22))</f>
         <v/>
       </c>
-      <c r="M22" s="12" t="n"/>
+      <c r="M22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="n"/>
@@ -2272,33 +1940,33 @@
       <c r="E23" s="8" t="n"/>
       <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="n"/>
-      <c r="H23" s="18" t="n"/>
-      <c r="I23" s="18" t="n"/>
+      <c r="H23" s="9" t="n"/>
+      <c r="I23" s="9" t="n"/>
       <c r="J23" s="8" t="n"/>
       <c r="K23" s="8" t="n"/>
-      <c r="L23" s="19">
+      <c r="L23" s="10">
         <f>IF(A23="","",DAYS(TODAY(),J23))</f>
         <v/>
       </c>
       <c r="M23" s="8" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n"/>
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="12" t="n"/>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="12" t="n"/>
-      <c r="F24" s="12" t="n"/>
-      <c r="G24" s="12" t="n"/>
-      <c r="H24" s="16" t="n"/>
-      <c r="I24" s="16" t="n"/>
-      <c r="J24" s="12" t="n"/>
-      <c r="K24" s="12" t="n"/>
-      <c r="L24" s="17">
+      <c r="A24" s="11" t="n"/>
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="11" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="11" t="n"/>
+      <c r="G24" s="11" t="n"/>
+      <c r="H24" s="12" t="n"/>
+      <c r="I24" s="12" t="n"/>
+      <c r="J24" s="11" t="n"/>
+      <c r="K24" s="11" t="n"/>
+      <c r="L24" s="13">
         <f>IF(A24="","",DAYS(TODAY(),J24))</f>
         <v/>
       </c>
-      <c r="M24" s="12" t="n"/>
+      <c r="M24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n"/>
@@ -2308,33 +1976,33 @@
       <c r="E25" s="8" t="n"/>
       <c r="F25" s="8" t="n"/>
       <c r="G25" s="8" t="n"/>
-      <c r="H25" s="18" t="n"/>
-      <c r="I25" s="18" t="n"/>
+      <c r="H25" s="9" t="n"/>
+      <c r="I25" s="9" t="n"/>
       <c r="J25" s="8" t="n"/>
       <c r="K25" s="8" t="n"/>
-      <c r="L25" s="19">
+      <c r="L25" s="10">
         <f>IF(A25="","",DAYS(TODAY(),J25))</f>
         <v/>
       </c>
       <c r="M25" s="8" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="n"/>
-      <c r="B26" s="12" t="n"/>
-      <c r="C26" s="12" t="n"/>
-      <c r="D26" s="12" t="n"/>
-      <c r="E26" s="12" t="n"/>
-      <c r="F26" s="12" t="n"/>
-      <c r="G26" s="12" t="n"/>
-      <c r="H26" s="16" t="n"/>
-      <c r="I26" s="16" t="n"/>
-      <c r="J26" s="12" t="n"/>
-      <c r="K26" s="12" t="n"/>
-      <c r="L26" s="17">
+      <c r="A26" s="11" t="n"/>
+      <c r="B26" s="11" t="n"/>
+      <c r="C26" s="11" t="n"/>
+      <c r="D26" s="11" t="n"/>
+      <c r="E26" s="11" t="n"/>
+      <c r="F26" s="11" t="n"/>
+      <c r="G26" s="11" t="n"/>
+      <c r="H26" s="12" t="n"/>
+      <c r="I26" s="12" t="n"/>
+      <c r="J26" s="11" t="n"/>
+      <c r="K26" s="11" t="n"/>
+      <c r="L26" s="13">
         <f>IF(A26="","",DAYS(TODAY(),J26))</f>
         <v/>
       </c>
-      <c r="M26" s="12" t="n"/>
+      <c r="M26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="n"/>
@@ -2344,33 +2012,33 @@
       <c r="E27" s="8" t="n"/>
       <c r="F27" s="8" t="n"/>
       <c r="G27" s="8" t="n"/>
-      <c r="H27" s="18" t="n"/>
-      <c r="I27" s="18" t="n"/>
+      <c r="H27" s="9" t="n"/>
+      <c r="I27" s="9" t="n"/>
       <c r="J27" s="8" t="n"/>
       <c r="K27" s="8" t="n"/>
-      <c r="L27" s="19">
+      <c r="L27" s="10">
         <f>IF(A27="","",DAYS(TODAY(),J27))</f>
         <v/>
       </c>
       <c r="M27" s="8" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n"/>
-      <c r="B28" s="12" t="n"/>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="12" t="n"/>
-      <c r="E28" s="12" t="n"/>
-      <c r="F28" s="12" t="n"/>
-      <c r="G28" s="12" t="n"/>
-      <c r="H28" s="16" t="n"/>
-      <c r="I28" s="16" t="n"/>
-      <c r="J28" s="12" t="n"/>
-      <c r="K28" s="12" t="n"/>
-      <c r="L28" s="17">
+      <c r="A28" s="11" t="n"/>
+      <c r="B28" s="11" t="n"/>
+      <c r="C28" s="11" t="n"/>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="11" t="n"/>
+      <c r="G28" s="11" t="n"/>
+      <c r="H28" s="12" t="n"/>
+      <c r="I28" s="12" t="n"/>
+      <c r="J28" s="11" t="n"/>
+      <c r="K28" s="11" t="n"/>
+      <c r="L28" s="13">
         <f>IF(A28="","",DAYS(TODAY(),J28))</f>
         <v/>
       </c>
-      <c r="M28" s="12" t="n"/>
+      <c r="M28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="n"/>
@@ -2380,33 +2048,33 @@
       <c r="E29" s="8" t="n"/>
       <c r="F29" s="8" t="n"/>
       <c r="G29" s="8" t="n"/>
-      <c r="H29" s="18" t="n"/>
-      <c r="I29" s="18" t="n"/>
+      <c r="H29" s="9" t="n"/>
+      <c r="I29" s="9" t="n"/>
       <c r="J29" s="8" t="n"/>
       <c r="K29" s="8" t="n"/>
-      <c r="L29" s="19">
+      <c r="L29" s="10">
         <f>IF(A29="","",DAYS(TODAY(),J29))</f>
         <v/>
       </c>
       <c r="M29" s="8" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n"/>
-      <c r="B30" s="12" t="n"/>
-      <c r="C30" s="12" t="n"/>
-      <c r="D30" s="12" t="n"/>
-      <c r="E30" s="12" t="n"/>
-      <c r="F30" s="12" t="n"/>
-      <c r="G30" s="12" t="n"/>
-      <c r="H30" s="16" t="n"/>
-      <c r="I30" s="16" t="n"/>
-      <c r="J30" s="12" t="n"/>
-      <c r="K30" s="12" t="n"/>
-      <c r="L30" s="17">
+      <c r="A30" s="11" t="n"/>
+      <c r="B30" s="11" t="n"/>
+      <c r="C30" s="11" t="n"/>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="11" t="n"/>
+      <c r="G30" s="11" t="n"/>
+      <c r="H30" s="12" t="n"/>
+      <c r="I30" s="12" t="n"/>
+      <c r="J30" s="11" t="n"/>
+      <c r="K30" s="11" t="n"/>
+      <c r="L30" s="13">
         <f>IF(A30="","",DAYS(TODAY(),J30))</f>
         <v/>
       </c>
-      <c r="M30" s="12" t="n"/>
+      <c r="M30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="n"/>
@@ -2416,33 +2084,33 @@
       <c r="E31" s="8" t="n"/>
       <c r="F31" s="8" t="n"/>
       <c r="G31" s="8" t="n"/>
-      <c r="H31" s="18" t="n"/>
-      <c r="I31" s="18" t="n"/>
+      <c r="H31" s="9" t="n"/>
+      <c r="I31" s="9" t="n"/>
       <c r="J31" s="8" t="n"/>
       <c r="K31" s="8" t="n"/>
-      <c r="L31" s="19">
+      <c r="L31" s="10">
         <f>IF(A31="","",DAYS(TODAY(),J31))</f>
         <v/>
       </c>
       <c r="M31" s="8" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="n"/>
-      <c r="B32" s="12" t="n"/>
-      <c r="C32" s="12" t="n"/>
-      <c r="D32" s="12" t="n"/>
-      <c r="E32" s="12" t="n"/>
-      <c r="F32" s="12" t="n"/>
-      <c r="G32" s="12" t="n"/>
-      <c r="H32" s="16" t="n"/>
-      <c r="I32" s="16" t="n"/>
-      <c r="J32" s="12" t="n"/>
-      <c r="K32" s="12" t="n"/>
-      <c r="L32" s="17">
+      <c r="A32" s="11" t="n"/>
+      <c r="B32" s="11" t="n"/>
+      <c r="C32" s="11" t="n"/>
+      <c r="D32" s="11" t="n"/>
+      <c r="E32" s="11" t="n"/>
+      <c r="F32" s="11" t="n"/>
+      <c r="G32" s="11" t="n"/>
+      <c r="H32" s="12" t="n"/>
+      <c r="I32" s="12" t="n"/>
+      <c r="J32" s="11" t="n"/>
+      <c r="K32" s="11" t="n"/>
+      <c r="L32" s="13">
         <f>IF(A32="","",DAYS(TODAY(),J32))</f>
         <v/>
       </c>
-      <c r="M32" s="12" t="n"/>
+      <c r="M32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="n"/>
@@ -2452,33 +2120,33 @@
       <c r="E33" s="8" t="n"/>
       <c r="F33" s="8" t="n"/>
       <c r="G33" s="8" t="n"/>
-      <c r="H33" s="18" t="n"/>
-      <c r="I33" s="18" t="n"/>
+      <c r="H33" s="9" t="n"/>
+      <c r="I33" s="9" t="n"/>
       <c r="J33" s="8" t="n"/>
       <c r="K33" s="8" t="n"/>
-      <c r="L33" s="19">
+      <c r="L33" s="10">
         <f>IF(A33="","",DAYS(TODAY(),J33))</f>
         <v/>
       </c>
       <c r="M33" s="8" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="n"/>
-      <c r="B34" s="12" t="n"/>
-      <c r="C34" s="12" t="n"/>
-      <c r="D34" s="12" t="n"/>
-      <c r="E34" s="12" t="n"/>
-      <c r="F34" s="12" t="n"/>
-      <c r="G34" s="12" t="n"/>
-      <c r="H34" s="16" t="n"/>
-      <c r="I34" s="16" t="n"/>
-      <c r="J34" s="12" t="n"/>
-      <c r="K34" s="12" t="n"/>
-      <c r="L34" s="17">
+      <c r="A34" s="11" t="n"/>
+      <c r="B34" s="11" t="n"/>
+      <c r="C34" s="11" t="n"/>
+      <c r="D34" s="11" t="n"/>
+      <c r="E34" s="11" t="n"/>
+      <c r="F34" s="11" t="n"/>
+      <c r="G34" s="11" t="n"/>
+      <c r="H34" s="12" t="n"/>
+      <c r="I34" s="12" t="n"/>
+      <c r="J34" s="11" t="n"/>
+      <c r="K34" s="11" t="n"/>
+      <c r="L34" s="13">
         <f>IF(A34="","",DAYS(TODAY(),J34))</f>
         <v/>
       </c>
-      <c r="M34" s="12" t="n"/>
+      <c r="M34" s="11" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="8" t="n"/>
@@ -2488,33 +2156,33 @@
       <c r="E35" s="8" t="n"/>
       <c r="F35" s="8" t="n"/>
       <c r="G35" s="8" t="n"/>
-      <c r="H35" s="18" t="n"/>
-      <c r="I35" s="18" t="n"/>
+      <c r="H35" s="9" t="n"/>
+      <c r="I35" s="9" t="n"/>
       <c r="J35" s="8" t="n"/>
       <c r="K35" s="8" t="n"/>
-      <c r="L35" s="19">
+      <c r="L35" s="10">
         <f>IF(A35="","",DAYS(TODAY(),J35))</f>
         <v/>
       </c>
       <c r="M35" s="8" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="n"/>
-      <c r="B36" s="12" t="n"/>
-      <c r="C36" s="12" t="n"/>
-      <c r="D36" s="12" t="n"/>
-      <c r="E36" s="12" t="n"/>
-      <c r="F36" s="12" t="n"/>
-      <c r="G36" s="12" t="n"/>
-      <c r="H36" s="16" t="n"/>
-      <c r="I36" s="16" t="n"/>
-      <c r="J36" s="12" t="n"/>
-      <c r="K36" s="12" t="n"/>
-      <c r="L36" s="17">
+      <c r="A36" s="11" t="n"/>
+      <c r="B36" s="11" t="n"/>
+      <c r="C36" s="11" t="n"/>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="11" t="n"/>
+      <c r="F36" s="11" t="n"/>
+      <c r="G36" s="11" t="n"/>
+      <c r="H36" s="12" t="n"/>
+      <c r="I36" s="12" t="n"/>
+      <c r="J36" s="11" t="n"/>
+      <c r="K36" s="11" t="n"/>
+      <c r="L36" s="13">
         <f>IF(A36="","",DAYS(TODAY(),J36))</f>
         <v/>
       </c>
-      <c r="M36" s="12" t="n"/>
+      <c r="M36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="n"/>
@@ -2524,33 +2192,33 @@
       <c r="E37" s="8" t="n"/>
       <c r="F37" s="8" t="n"/>
       <c r="G37" s="8" t="n"/>
-      <c r="H37" s="18" t="n"/>
-      <c r="I37" s="18" t="n"/>
+      <c r="H37" s="9" t="n"/>
+      <c r="I37" s="9" t="n"/>
       <c r="J37" s="8" t="n"/>
       <c r="K37" s="8" t="n"/>
-      <c r="L37" s="19">
+      <c r="L37" s="10">
         <f>IF(A37="","",DAYS(TODAY(),J37))</f>
         <v/>
       </c>
       <c r="M37" s="8" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="12" t="n"/>
-      <c r="B38" s="12" t="n"/>
-      <c r="C38" s="12" t="n"/>
-      <c r="D38" s="12" t="n"/>
-      <c r="E38" s="12" t="n"/>
-      <c r="F38" s="12" t="n"/>
-      <c r="G38" s="12" t="n"/>
-      <c r="H38" s="16" t="n"/>
-      <c r="I38" s="16" t="n"/>
-      <c r="J38" s="12" t="n"/>
-      <c r="K38" s="12" t="n"/>
-      <c r="L38" s="17">
+      <c r="A38" s="11" t="n"/>
+      <c r="B38" s="11" t="n"/>
+      <c r="C38" s="11" t="n"/>
+      <c r="D38" s="11" t="n"/>
+      <c r="E38" s="11" t="n"/>
+      <c r="F38" s="11" t="n"/>
+      <c r="G38" s="11" t="n"/>
+      <c r="H38" s="12" t="n"/>
+      <c r="I38" s="12" t="n"/>
+      <c r="J38" s="11" t="n"/>
+      <c r="K38" s="11" t="n"/>
+      <c r="L38" s="13">
         <f>IF(A38="","",DAYS(TODAY(),J38))</f>
         <v/>
       </c>
-      <c r="M38" s="12" t="n"/>
+      <c r="M38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="n"/>
@@ -2560,33 +2228,33 @@
       <c r="E39" s="8" t="n"/>
       <c r="F39" s="8" t="n"/>
       <c r="G39" s="8" t="n"/>
-      <c r="H39" s="18" t="n"/>
-      <c r="I39" s="18" t="n"/>
+      <c r="H39" s="9" t="n"/>
+      <c r="I39" s="9" t="n"/>
       <c r="J39" s="8" t="n"/>
       <c r="K39" s="8" t="n"/>
-      <c r="L39" s="19">
+      <c r="L39" s="10">
         <f>IF(A39="","",DAYS(TODAY(),J39))</f>
         <v/>
       </c>
       <c r="M39" s="8" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="12" t="n"/>
-      <c r="B40" s="12" t="n"/>
-      <c r="C40" s="12" t="n"/>
-      <c r="D40" s="12" t="n"/>
-      <c r="E40" s="12" t="n"/>
-      <c r="F40" s="12" t="n"/>
-      <c r="G40" s="12" t="n"/>
-      <c r="H40" s="16" t="n"/>
-      <c r="I40" s="16" t="n"/>
-      <c r="J40" s="12" t="n"/>
-      <c r="K40" s="12" t="n"/>
-      <c r="L40" s="17">
+      <c r="A40" s="11" t="n"/>
+      <c r="B40" s="11" t="n"/>
+      <c r="C40" s="11" t="n"/>
+      <c r="D40" s="11" t="n"/>
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="11" t="n"/>
+      <c r="G40" s="11" t="n"/>
+      <c r="H40" s="12" t="n"/>
+      <c r="I40" s="12" t="n"/>
+      <c r="J40" s="11" t="n"/>
+      <c r="K40" s="11" t="n"/>
+      <c r="L40" s="13">
         <f>IF(A40="","",DAYS(TODAY(),J40))</f>
         <v/>
       </c>
-      <c r="M40" s="12" t="n"/>
+      <c r="M40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="8" t="n"/>
@@ -2596,33 +2264,33 @@
       <c r="E41" s="8" t="n"/>
       <c r="F41" s="8" t="n"/>
       <c r="G41" s="8" t="n"/>
-      <c r="H41" s="18" t="n"/>
-      <c r="I41" s="18" t="n"/>
+      <c r="H41" s="9" t="n"/>
+      <c r="I41" s="9" t="n"/>
       <c r="J41" s="8" t="n"/>
       <c r="K41" s="8" t="n"/>
-      <c r="L41" s="19">
+      <c r="L41" s="10">
         <f>IF(A41="","",DAYS(TODAY(),J41))</f>
         <v/>
       </c>
       <c r="M41" s="8" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="12" t="n"/>
-      <c r="B42" s="12" t="n"/>
-      <c r="C42" s="12" t="n"/>
-      <c r="D42" s="12" t="n"/>
-      <c r="E42" s="12" t="n"/>
-      <c r="F42" s="12" t="n"/>
-      <c r="G42" s="12" t="n"/>
-      <c r="H42" s="16" t="n"/>
-      <c r="I42" s="16" t="n"/>
-      <c r="J42" s="12" t="n"/>
-      <c r="K42" s="12" t="n"/>
-      <c r="L42" s="17">
+      <c r="A42" s="11" t="n"/>
+      <c r="B42" s="11" t="n"/>
+      <c r="C42" s="11" t="n"/>
+      <c r="D42" s="11" t="n"/>
+      <c r="E42" s="11" t="n"/>
+      <c r="F42" s="11" t="n"/>
+      <c r="G42" s="11" t="n"/>
+      <c r="H42" s="12" t="n"/>
+      <c r="I42" s="12" t="n"/>
+      <c r="J42" s="11" t="n"/>
+      <c r="K42" s="11" t="n"/>
+      <c r="L42" s="13">
         <f>IF(A42="","",DAYS(TODAY(),J42))</f>
         <v/>
       </c>
-      <c r="M42" s="12" t="n"/>
+      <c r="M42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="8" t="n"/>
@@ -2632,33 +2300,33 @@
       <c r="E43" s="8" t="n"/>
       <c r="F43" s="8" t="n"/>
       <c r="G43" s="8" t="n"/>
-      <c r="H43" s="18" t="n"/>
-      <c r="I43" s="18" t="n"/>
+      <c r="H43" s="9" t="n"/>
+      <c r="I43" s="9" t="n"/>
       <c r="J43" s="8" t="n"/>
       <c r="K43" s="8" t="n"/>
-      <c r="L43" s="19">
+      <c r="L43" s="10">
         <f>IF(A43="","",DAYS(TODAY(),J43))</f>
         <v/>
       </c>
       <c r="M43" s="8" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="n"/>
-      <c r="B44" s="12" t="n"/>
-      <c r="C44" s="12" t="n"/>
-      <c r="D44" s="12" t="n"/>
-      <c r="E44" s="12" t="n"/>
-      <c r="F44" s="12" t="n"/>
-      <c r="G44" s="12" t="n"/>
-      <c r="H44" s="16" t="n"/>
-      <c r="I44" s="16" t="n"/>
-      <c r="J44" s="12" t="n"/>
-      <c r="K44" s="12" t="n"/>
-      <c r="L44" s="17">
+      <c r="A44" s="11" t="n"/>
+      <c r="B44" s="11" t="n"/>
+      <c r="C44" s="11" t="n"/>
+      <c r="D44" s="11" t="n"/>
+      <c r="E44" s="11" t="n"/>
+      <c r="F44" s="11" t="n"/>
+      <c r="G44" s="11" t="n"/>
+      <c r="H44" s="12" t="n"/>
+      <c r="I44" s="12" t="n"/>
+      <c r="J44" s="11" t="n"/>
+      <c r="K44" s="11" t="n"/>
+      <c r="L44" s="13">
         <f>IF(A44="","",DAYS(TODAY(),J44))</f>
         <v/>
       </c>
-      <c r="M44" s="12" t="n"/>
+      <c r="M44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="n"/>
@@ -2668,33 +2336,33 @@
       <c r="E45" s="8" t="n"/>
       <c r="F45" s="8" t="n"/>
       <c r="G45" s="8" t="n"/>
-      <c r="H45" s="18" t="n"/>
-      <c r="I45" s="18" t="n"/>
+      <c r="H45" s="9" t="n"/>
+      <c r="I45" s="9" t="n"/>
       <c r="J45" s="8" t="n"/>
       <c r="K45" s="8" t="n"/>
-      <c r="L45" s="19">
+      <c r="L45" s="10">
         <f>IF(A45="","",DAYS(TODAY(),J45))</f>
         <v/>
       </c>
       <c r="M45" s="8" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="12" t="n"/>
-      <c r="B46" s="12" t="n"/>
-      <c r="C46" s="12" t="n"/>
-      <c r="D46" s="12" t="n"/>
-      <c r="E46" s="12" t="n"/>
-      <c r="F46" s="12" t="n"/>
-      <c r="G46" s="12" t="n"/>
-      <c r="H46" s="16" t="n"/>
-      <c r="I46" s="16" t="n"/>
-      <c r="J46" s="12" t="n"/>
-      <c r="K46" s="12" t="n"/>
-      <c r="L46" s="17">
+      <c r="A46" s="11" t="n"/>
+      <c r="B46" s="11" t="n"/>
+      <c r="C46" s="11" t="n"/>
+      <c r="D46" s="11" t="n"/>
+      <c r="E46" s="11" t="n"/>
+      <c r="F46" s="11" t="n"/>
+      <c r="G46" s="11" t="n"/>
+      <c r="H46" s="12" t="n"/>
+      <c r="I46" s="12" t="n"/>
+      <c r="J46" s="11" t="n"/>
+      <c r="K46" s="11" t="n"/>
+      <c r="L46" s="13">
         <f>IF(A46="","",DAYS(TODAY(),J46))</f>
         <v/>
       </c>
-      <c r="M46" s="12" t="n"/>
+      <c r="M46" s="11" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="8" t="n"/>
@@ -2704,33 +2372,33 @@
       <c r="E47" s="8" t="n"/>
       <c r="F47" s="8" t="n"/>
       <c r="G47" s="8" t="n"/>
-      <c r="H47" s="18" t="n"/>
-      <c r="I47" s="18" t="n"/>
+      <c r="H47" s="9" t="n"/>
+      <c r="I47" s="9" t="n"/>
       <c r="J47" s="8" t="n"/>
       <c r="K47" s="8" t="n"/>
-      <c r="L47" s="19">
+      <c r="L47" s="10">
         <f>IF(A47="","",DAYS(TODAY(),J47))</f>
         <v/>
       </c>
       <c r="M47" s="8" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="12" t="n"/>
-      <c r="B48" s="12" t="n"/>
-      <c r="C48" s="12" t="n"/>
-      <c r="D48" s="12" t="n"/>
-      <c r="E48" s="12" t="n"/>
-      <c r="F48" s="12" t="n"/>
-      <c r="G48" s="12" t="n"/>
-      <c r="H48" s="16" t="n"/>
-      <c r="I48" s="16" t="n"/>
-      <c r="J48" s="12" t="n"/>
-      <c r="K48" s="12" t="n"/>
-      <c r="L48" s="17">
+      <c r="A48" s="11" t="n"/>
+      <c r="B48" s="11" t="n"/>
+      <c r="C48" s="11" t="n"/>
+      <c r="D48" s="11" t="n"/>
+      <c r="E48" s="11" t="n"/>
+      <c r="F48" s="11" t="n"/>
+      <c r="G48" s="11" t="n"/>
+      <c r="H48" s="12" t="n"/>
+      <c r="I48" s="12" t="n"/>
+      <c r="J48" s="11" t="n"/>
+      <c r="K48" s="11" t="n"/>
+      <c r="L48" s="13">
         <f>IF(A48="","",DAYS(TODAY(),J48))</f>
         <v/>
       </c>
-      <c r="M48" s="12" t="n"/>
+      <c r="M48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="8" t="n"/>
@@ -2740,33 +2408,33 @@
       <c r="E49" s="8" t="n"/>
       <c r="F49" s="8" t="n"/>
       <c r="G49" s="8" t="n"/>
-      <c r="H49" s="18" t="n"/>
-      <c r="I49" s="18" t="n"/>
+      <c r="H49" s="9" t="n"/>
+      <c r="I49" s="9" t="n"/>
       <c r="J49" s="8" t="n"/>
       <c r="K49" s="8" t="n"/>
-      <c r="L49" s="19">
+      <c r="L49" s="10">
         <f>IF(A49="","",DAYS(TODAY(),J49))</f>
         <v/>
       </c>
       <c r="M49" s="8" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="12" t="n"/>
-      <c r="B50" s="12" t="n"/>
-      <c r="C50" s="12" t="n"/>
-      <c r="D50" s="12" t="n"/>
-      <c r="E50" s="12" t="n"/>
-      <c r="F50" s="12" t="n"/>
-      <c r="G50" s="12" t="n"/>
-      <c r="H50" s="16" t="n"/>
-      <c r="I50" s="16" t="n"/>
-      <c r="J50" s="12" t="n"/>
-      <c r="K50" s="12" t="n"/>
-      <c r="L50" s="17">
+      <c r="A50" s="11" t="n"/>
+      <c r="B50" s="11" t="n"/>
+      <c r="C50" s="11" t="n"/>
+      <c r="D50" s="11" t="n"/>
+      <c r="E50" s="11" t="n"/>
+      <c r="F50" s="11" t="n"/>
+      <c r="G50" s="11" t="n"/>
+      <c r="H50" s="12" t="n"/>
+      <c r="I50" s="12" t="n"/>
+      <c r="J50" s="11" t="n"/>
+      <c r="K50" s="11" t="n"/>
+      <c r="L50" s="13">
         <f>IF(A50="","",DAYS(TODAY(),J50))</f>
         <v/>
       </c>
-      <c r="M50" s="12" t="n"/>
+      <c r="M50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="n"/>
@@ -2776,33 +2444,33 @@
       <c r="E51" s="8" t="n"/>
       <c r="F51" s="8" t="n"/>
       <c r="G51" s="8" t="n"/>
-      <c r="H51" s="18" t="n"/>
-      <c r="I51" s="18" t="n"/>
+      <c r="H51" s="9" t="n"/>
+      <c r="I51" s="9" t="n"/>
       <c r="J51" s="8" t="n"/>
       <c r="K51" s="8" t="n"/>
-      <c r="L51" s="19">
+      <c r="L51" s="10">
         <f>IF(A51="","",DAYS(TODAY(),J51))</f>
         <v/>
       </c>
       <c r="M51" s="8" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="12" t="n"/>
-      <c r="B52" s="12" t="n"/>
-      <c r="C52" s="12" t="n"/>
-      <c r="D52" s="12" t="n"/>
-      <c r="E52" s="12" t="n"/>
-      <c r="F52" s="12" t="n"/>
-      <c r="G52" s="12" t="n"/>
-      <c r="H52" s="16" t="n"/>
-      <c r="I52" s="16" t="n"/>
-      <c r="J52" s="12" t="n"/>
-      <c r="K52" s="12" t="n"/>
-      <c r="L52" s="17">
+      <c r="A52" s="11" t="n"/>
+      <c r="B52" s="11" t="n"/>
+      <c r="C52" s="11" t="n"/>
+      <c r="D52" s="11" t="n"/>
+      <c r="E52" s="11" t="n"/>
+      <c r="F52" s="11" t="n"/>
+      <c r="G52" s="11" t="n"/>
+      <c r="H52" s="12" t="n"/>
+      <c r="I52" s="12" t="n"/>
+      <c r="J52" s="11" t="n"/>
+      <c r="K52" s="11" t="n"/>
+      <c r="L52" s="13">
         <f>IF(A52="","",DAYS(TODAY(),J52))</f>
         <v/>
       </c>
-      <c r="M52" s="12" t="n"/>
+      <c r="M52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="8" t="n"/>
@@ -2812,33 +2480,33 @@
       <c r="E53" s="8" t="n"/>
       <c r="F53" s="8" t="n"/>
       <c r="G53" s="8" t="n"/>
-      <c r="H53" s="18" t="n"/>
-      <c r="I53" s="18" t="n"/>
+      <c r="H53" s="9" t="n"/>
+      <c r="I53" s="9" t="n"/>
       <c r="J53" s="8" t="n"/>
       <c r="K53" s="8" t="n"/>
-      <c r="L53" s="19">
+      <c r="L53" s="10">
         <f>IF(A53="","",DAYS(TODAY(),J53))</f>
         <v/>
       </c>
       <c r="M53" s="8" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="12" t="n"/>
-      <c r="B54" s="12" t="n"/>
-      <c r="C54" s="12" t="n"/>
-      <c r="D54" s="12" t="n"/>
-      <c r="E54" s="12" t="n"/>
-      <c r="F54" s="12" t="n"/>
-      <c r="G54" s="12" t="n"/>
-      <c r="H54" s="16" t="n"/>
-      <c r="I54" s="16" t="n"/>
-      <c r="J54" s="12" t="n"/>
-      <c r="K54" s="12" t="n"/>
-      <c r="L54" s="17">
+      <c r="A54" s="11" t="n"/>
+      <c r="B54" s="11" t="n"/>
+      <c r="C54" s="11" t="n"/>
+      <c r="D54" s="11" t="n"/>
+      <c r="E54" s="11" t="n"/>
+      <c r="F54" s="11" t="n"/>
+      <c r="G54" s="11" t="n"/>
+      <c r="H54" s="12" t="n"/>
+      <c r="I54" s="12" t="n"/>
+      <c r="J54" s="11" t="n"/>
+      <c r="K54" s="11" t="n"/>
+      <c r="L54" s="13">
         <f>IF(A54="","",DAYS(TODAY(),J54))</f>
         <v/>
       </c>
-      <c r="M54" s="12" t="n"/>
+      <c r="M54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="8" t="n"/>
@@ -2848,33 +2516,33 @@
       <c r="E55" s="8" t="n"/>
       <c r="F55" s="8" t="n"/>
       <c r="G55" s="8" t="n"/>
-      <c r="H55" s="18" t="n"/>
-      <c r="I55" s="18" t="n"/>
+      <c r="H55" s="9" t="n"/>
+      <c r="I55" s="9" t="n"/>
       <c r="J55" s="8" t="n"/>
       <c r="K55" s="8" t="n"/>
-      <c r="L55" s="19">
+      <c r="L55" s="10">
         <f>IF(A55="","",DAYS(TODAY(),J55))</f>
         <v/>
       </c>
       <c r="M55" s="8" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="12" t="n"/>
-      <c r="B56" s="12" t="n"/>
-      <c r="C56" s="12" t="n"/>
-      <c r="D56" s="12" t="n"/>
-      <c r="E56" s="12" t="n"/>
-      <c r="F56" s="12" t="n"/>
-      <c r="G56" s="12" t="n"/>
-      <c r="H56" s="16" t="n"/>
-      <c r="I56" s="16" t="n"/>
-      <c r="J56" s="12" t="n"/>
-      <c r="K56" s="12" t="n"/>
-      <c r="L56" s="17">
+      <c r="A56" s="11" t="n"/>
+      <c r="B56" s="11" t="n"/>
+      <c r="C56" s="11" t="n"/>
+      <c r="D56" s="11" t="n"/>
+      <c r="E56" s="11" t="n"/>
+      <c r="F56" s="11" t="n"/>
+      <c r="G56" s="11" t="n"/>
+      <c r="H56" s="12" t="n"/>
+      <c r="I56" s="12" t="n"/>
+      <c r="J56" s="11" t="n"/>
+      <c r="K56" s="11" t="n"/>
+      <c r="L56" s="13">
         <f>IF(A56="","",DAYS(TODAY(),J56))</f>
         <v/>
       </c>
-      <c r="M56" s="12" t="n"/>
+      <c r="M56" s="11" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="8" t="n"/>
@@ -2884,33 +2552,33 @@
       <c r="E57" s="8" t="n"/>
       <c r="F57" s="8" t="n"/>
       <c r="G57" s="8" t="n"/>
-      <c r="H57" s="18" t="n"/>
-      <c r="I57" s="18" t="n"/>
+      <c r="H57" s="9" t="n"/>
+      <c r="I57" s="9" t="n"/>
       <c r="J57" s="8" t="n"/>
       <c r="K57" s="8" t="n"/>
-      <c r="L57" s="19">
+      <c r="L57" s="10">
         <f>IF(A57="","",DAYS(TODAY(),J57))</f>
         <v/>
       </c>
       <c r="M57" s="8" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="12" t="n"/>
-      <c r="B58" s="12" t="n"/>
-      <c r="C58" s="12" t="n"/>
-      <c r="D58" s="12" t="n"/>
-      <c r="E58" s="12" t="n"/>
-      <c r="F58" s="12" t="n"/>
-      <c r="G58" s="12" t="n"/>
-      <c r="H58" s="16" t="n"/>
-      <c r="I58" s="16" t="n"/>
-      <c r="J58" s="12" t="n"/>
-      <c r="K58" s="12" t="n"/>
-      <c r="L58" s="17">
+      <c r="A58" s="11" t="n"/>
+      <c r="B58" s="11" t="n"/>
+      <c r="C58" s="11" t="n"/>
+      <c r="D58" s="11" t="n"/>
+      <c r="E58" s="11" t="n"/>
+      <c r="F58" s="11" t="n"/>
+      <c r="G58" s="11" t="n"/>
+      <c r="H58" s="12" t="n"/>
+      <c r="I58" s="12" t="n"/>
+      <c r="J58" s="11" t="n"/>
+      <c r="K58" s="11" t="n"/>
+      <c r="L58" s="13">
         <f>IF(A58="","",DAYS(TODAY(),J58))</f>
         <v/>
       </c>
-      <c r="M58" s="12" t="n"/>
+      <c r="M58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n"/>
@@ -2920,33 +2588,33 @@
       <c r="E59" s="8" t="n"/>
       <c r="F59" s="8" t="n"/>
       <c r="G59" s="8" t="n"/>
-      <c r="H59" s="18" t="n"/>
-      <c r="I59" s="18" t="n"/>
+      <c r="H59" s="9" t="n"/>
+      <c r="I59" s="9" t="n"/>
       <c r="J59" s="8" t="n"/>
       <c r="K59" s="8" t="n"/>
-      <c r="L59" s="19">
+      <c r="L59" s="10">
         <f>IF(A59="","",DAYS(TODAY(),J59))</f>
         <v/>
       </c>
       <c r="M59" s="8" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="12" t="n"/>
-      <c r="B60" s="12" t="n"/>
-      <c r="C60" s="12" t="n"/>
-      <c r="D60" s="12" t="n"/>
-      <c r="E60" s="12" t="n"/>
-      <c r="F60" s="12" t="n"/>
-      <c r="G60" s="12" t="n"/>
-      <c r="H60" s="16" t="n"/>
-      <c r="I60" s="16" t="n"/>
-      <c r="J60" s="12" t="n"/>
-      <c r="K60" s="12" t="n"/>
-      <c r="L60" s="17">
+      <c r="A60" s="11" t="n"/>
+      <c r="B60" s="11" t="n"/>
+      <c r="C60" s="11" t="n"/>
+      <c r="D60" s="11" t="n"/>
+      <c r="E60" s="11" t="n"/>
+      <c r="F60" s="11" t="n"/>
+      <c r="G60" s="11" t="n"/>
+      <c r="H60" s="12" t="n"/>
+      <c r="I60" s="12" t="n"/>
+      <c r="J60" s="11" t="n"/>
+      <c r="K60" s="11" t="n"/>
+      <c r="L60" s="13">
         <f>IF(A60="","",DAYS(TODAY(),J60))</f>
         <v/>
       </c>
-      <c r="M60" s="12" t="n"/>
+      <c r="M60" s="11" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="8" t="n"/>
@@ -2956,33 +2624,33 @@
       <c r="E61" s="8" t="n"/>
       <c r="F61" s="8" t="n"/>
       <c r="G61" s="8" t="n"/>
-      <c r="H61" s="18" t="n"/>
-      <c r="I61" s="18" t="n"/>
+      <c r="H61" s="9" t="n"/>
+      <c r="I61" s="9" t="n"/>
       <c r="J61" s="8" t="n"/>
       <c r="K61" s="8" t="n"/>
-      <c r="L61" s="19">
+      <c r="L61" s="10">
         <f>IF(A61="","",DAYS(TODAY(),J61))</f>
         <v/>
       </c>
       <c r="M61" s="8" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="12" t="n"/>
-      <c r="B62" s="12" t="n"/>
-      <c r="C62" s="12" t="n"/>
-      <c r="D62" s="12" t="n"/>
-      <c r="E62" s="12" t="n"/>
-      <c r="F62" s="12" t="n"/>
-      <c r="G62" s="12" t="n"/>
-      <c r="H62" s="16" t="n"/>
-      <c r="I62" s="16" t="n"/>
-      <c r="J62" s="12" t="n"/>
-      <c r="K62" s="12" t="n"/>
-      <c r="L62" s="17">
+      <c r="A62" s="11" t="n"/>
+      <c r="B62" s="11" t="n"/>
+      <c r="C62" s="11" t="n"/>
+      <c r="D62" s="11" t="n"/>
+      <c r="E62" s="11" t="n"/>
+      <c r="F62" s="11" t="n"/>
+      <c r="G62" s="11" t="n"/>
+      <c r="H62" s="12" t="n"/>
+      <c r="I62" s="12" t="n"/>
+      <c r="J62" s="11" t="n"/>
+      <c r="K62" s="11" t="n"/>
+      <c r="L62" s="13">
         <f>IF(A62="","",DAYS(TODAY(),J62))</f>
         <v/>
       </c>
-      <c r="M62" s="12" t="n"/>
+      <c r="M62" s="11" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="8" t="n"/>
@@ -2992,33 +2660,33 @@
       <c r="E63" s="8" t="n"/>
       <c r="F63" s="8" t="n"/>
       <c r="G63" s="8" t="n"/>
-      <c r="H63" s="18" t="n"/>
-      <c r="I63" s="18" t="n"/>
+      <c r="H63" s="9" t="n"/>
+      <c r="I63" s="9" t="n"/>
       <c r="J63" s="8" t="n"/>
       <c r="K63" s="8" t="n"/>
-      <c r="L63" s="19">
+      <c r="L63" s="10">
         <f>IF(A63="","",DAYS(TODAY(),J63))</f>
         <v/>
       </c>
       <c r="M63" s="8" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="12" t="n"/>
-      <c r="B64" s="12" t="n"/>
-      <c r="C64" s="12" t="n"/>
-      <c r="D64" s="12" t="n"/>
-      <c r="E64" s="12" t="n"/>
-      <c r="F64" s="12" t="n"/>
-      <c r="G64" s="12" t="n"/>
-      <c r="H64" s="16" t="n"/>
-      <c r="I64" s="16" t="n"/>
-      <c r="J64" s="12" t="n"/>
-      <c r="K64" s="12" t="n"/>
-      <c r="L64" s="17">
+      <c r="A64" s="11" t="n"/>
+      <c r="B64" s="11" t="n"/>
+      <c r="C64" s="11" t="n"/>
+      <c r="D64" s="11" t="n"/>
+      <c r="E64" s="11" t="n"/>
+      <c r="F64" s="11" t="n"/>
+      <c r="G64" s="11" t="n"/>
+      <c r="H64" s="12" t="n"/>
+      <c r="I64" s="12" t="n"/>
+      <c r="J64" s="11" t="n"/>
+      <c r="K64" s="11" t="n"/>
+      <c r="L64" s="13">
         <f>IF(A64="","",DAYS(TODAY(),J64))</f>
         <v/>
       </c>
-      <c r="M64" s="12" t="n"/>
+      <c r="M64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="8" t="n"/>
@@ -3028,33 +2696,33 @@
       <c r="E65" s="8" t="n"/>
       <c r="F65" s="8" t="n"/>
       <c r="G65" s="8" t="n"/>
-      <c r="H65" s="18" t="n"/>
-      <c r="I65" s="18" t="n"/>
+      <c r="H65" s="9" t="n"/>
+      <c r="I65" s="9" t="n"/>
       <c r="J65" s="8" t="n"/>
       <c r="K65" s="8" t="n"/>
-      <c r="L65" s="19">
+      <c r="L65" s="10">
         <f>IF(A65="","",DAYS(TODAY(),J65))</f>
         <v/>
       </c>
       <c r="M65" s="8" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="12" t="n"/>
-      <c r="B66" s="12" t="n"/>
-      <c r="C66" s="12" t="n"/>
-      <c r="D66" s="12" t="n"/>
-      <c r="E66" s="12" t="n"/>
-      <c r="F66" s="12" t="n"/>
-      <c r="G66" s="12" t="n"/>
-      <c r="H66" s="16" t="n"/>
-      <c r="I66" s="16" t="n"/>
-      <c r="J66" s="12" t="n"/>
-      <c r="K66" s="12" t="n"/>
-      <c r="L66" s="17">
+      <c r="A66" s="11" t="n"/>
+      <c r="B66" s="11" t="n"/>
+      <c r="C66" s="11" t="n"/>
+      <c r="D66" s="11" t="n"/>
+      <c r="E66" s="11" t="n"/>
+      <c r="F66" s="11" t="n"/>
+      <c r="G66" s="11" t="n"/>
+      <c r="H66" s="12" t="n"/>
+      <c r="I66" s="12" t="n"/>
+      <c r="J66" s="11" t="n"/>
+      <c r="K66" s="11" t="n"/>
+      <c r="L66" s="13">
         <f>IF(A66="","",DAYS(TODAY(),J66))</f>
         <v/>
       </c>
-      <c r="M66" s="12" t="n"/>
+      <c r="M66" s="11" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="8" t="n"/>
@@ -3064,33 +2732,33 @@
       <c r="E67" s="8" t="n"/>
       <c r="F67" s="8" t="n"/>
       <c r="G67" s="8" t="n"/>
-      <c r="H67" s="18" t="n"/>
-      <c r="I67" s="18" t="n"/>
+      <c r="H67" s="9" t="n"/>
+      <c r="I67" s="9" t="n"/>
       <c r="J67" s="8" t="n"/>
       <c r="K67" s="8" t="n"/>
-      <c r="L67" s="19">
+      <c r="L67" s="10">
         <f>IF(A67="","",DAYS(TODAY(),J67))</f>
         <v/>
       </c>
       <c r="M67" s="8" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="12" t="n"/>
-      <c r="B68" s="12" t="n"/>
-      <c r="C68" s="12" t="n"/>
-      <c r="D68" s="12" t="n"/>
-      <c r="E68" s="12" t="n"/>
-      <c r="F68" s="12" t="n"/>
-      <c r="G68" s="12" t="n"/>
-      <c r="H68" s="16" t="n"/>
-      <c r="I68" s="16" t="n"/>
-      <c r="J68" s="12" t="n"/>
-      <c r="K68" s="12" t="n"/>
-      <c r="L68" s="17">
+      <c r="A68" s="11" t="n"/>
+      <c r="B68" s="11" t="n"/>
+      <c r="C68" s="11" t="n"/>
+      <c r="D68" s="11" t="n"/>
+      <c r="E68" s="11" t="n"/>
+      <c r="F68" s="11" t="n"/>
+      <c r="G68" s="11" t="n"/>
+      <c r="H68" s="12" t="n"/>
+      <c r="I68" s="12" t="n"/>
+      <c r="J68" s="11" t="n"/>
+      <c r="K68" s="11" t="n"/>
+      <c r="L68" s="13">
         <f>IF(A68="","",DAYS(TODAY(),J68))</f>
         <v/>
       </c>
-      <c r="M68" s="12" t="n"/>
+      <c r="M68" s="11" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="8" t="n"/>
@@ -3100,33 +2768,33 @@
       <c r="E69" s="8" t="n"/>
       <c r="F69" s="8" t="n"/>
       <c r="G69" s="8" t="n"/>
-      <c r="H69" s="18" t="n"/>
-      <c r="I69" s="18" t="n"/>
+      <c r="H69" s="9" t="n"/>
+      <c r="I69" s="9" t="n"/>
       <c r="J69" s="8" t="n"/>
       <c r="K69" s="8" t="n"/>
-      <c r="L69" s="19">
+      <c r="L69" s="10">
         <f>IF(A69="","",DAYS(TODAY(),J69))</f>
         <v/>
       </c>
       <c r="M69" s="8" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="12" t="n"/>
-      <c r="B70" s="12" t="n"/>
-      <c r="C70" s="12" t="n"/>
-      <c r="D70" s="12" t="n"/>
-      <c r="E70" s="12" t="n"/>
-      <c r="F70" s="12" t="n"/>
-      <c r="G70" s="12" t="n"/>
-      <c r="H70" s="16" t="n"/>
-      <c r="I70" s="16" t="n"/>
-      <c r="J70" s="12" t="n"/>
-      <c r="K70" s="12" t="n"/>
-      <c r="L70" s="17">
+      <c r="A70" s="11" t="n"/>
+      <c r="B70" s="11" t="n"/>
+      <c r="C70" s="11" t="n"/>
+      <c r="D70" s="11" t="n"/>
+      <c r="E70" s="11" t="n"/>
+      <c r="F70" s="11" t="n"/>
+      <c r="G70" s="11" t="n"/>
+      <c r="H70" s="12" t="n"/>
+      <c r="I70" s="12" t="n"/>
+      <c r="J70" s="11" t="n"/>
+      <c r="K70" s="11" t="n"/>
+      <c r="L70" s="13">
         <f>IF(A70="","",DAYS(TODAY(),J70))</f>
         <v/>
       </c>
-      <c r="M70" s="12" t="n"/>
+      <c r="M70" s="11" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="8" t="n"/>
@@ -3136,33 +2804,33 @@
       <c r="E71" s="8" t="n"/>
       <c r="F71" s="8" t="n"/>
       <c r="G71" s="8" t="n"/>
-      <c r="H71" s="18" t="n"/>
-      <c r="I71" s="18" t="n"/>
+      <c r="H71" s="9" t="n"/>
+      <c r="I71" s="9" t="n"/>
       <c r="J71" s="8" t="n"/>
       <c r="K71" s="8" t="n"/>
-      <c r="L71" s="19">
+      <c r="L71" s="10">
         <f>IF(A71="","",DAYS(TODAY(),J71))</f>
         <v/>
       </c>
       <c r="M71" s="8" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="12" t="n"/>
-      <c r="B72" s="12" t="n"/>
-      <c r="C72" s="12" t="n"/>
-      <c r="D72" s="12" t="n"/>
-      <c r="E72" s="12" t="n"/>
-      <c r="F72" s="12" t="n"/>
-      <c r="G72" s="12" t="n"/>
-      <c r="H72" s="16" t="n"/>
-      <c r="I72" s="16" t="n"/>
-      <c r="J72" s="12" t="n"/>
-      <c r="K72" s="12" t="n"/>
-      <c r="L72" s="17">
+      <c r="A72" s="11" t="n"/>
+      <c r="B72" s="11" t="n"/>
+      <c r="C72" s="11" t="n"/>
+      <c r="D72" s="11" t="n"/>
+      <c r="E72" s="11" t="n"/>
+      <c r="F72" s="11" t="n"/>
+      <c r="G72" s="11" t="n"/>
+      <c r="H72" s="12" t="n"/>
+      <c r="I72" s="12" t="n"/>
+      <c r="J72" s="11" t="n"/>
+      <c r="K72" s="11" t="n"/>
+      <c r="L72" s="13">
         <f>IF(A72="","",DAYS(TODAY(),J72))</f>
         <v/>
       </c>
-      <c r="M72" s="12" t="n"/>
+      <c r="M72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="8" t="n"/>
@@ -3172,33 +2840,33 @@
       <c r="E73" s="8" t="n"/>
       <c r="F73" s="8" t="n"/>
       <c r="G73" s="8" t="n"/>
-      <c r="H73" s="18" t="n"/>
-      <c r="I73" s="18" t="n"/>
+      <c r="H73" s="9" t="n"/>
+      <c r="I73" s="9" t="n"/>
       <c r="J73" s="8" t="n"/>
       <c r="K73" s="8" t="n"/>
-      <c r="L73" s="19">
+      <c r="L73" s="10">
         <f>IF(A73="","",DAYS(TODAY(),J73))</f>
         <v/>
       </c>
       <c r="M73" s="8" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="12" t="n"/>
-      <c r="B74" s="12" t="n"/>
-      <c r="C74" s="12" t="n"/>
-      <c r="D74" s="12" t="n"/>
-      <c r="E74" s="12" t="n"/>
-      <c r="F74" s="12" t="n"/>
-      <c r="G74" s="12" t="n"/>
-      <c r="H74" s="16" t="n"/>
-      <c r="I74" s="16" t="n"/>
-      <c r="J74" s="12" t="n"/>
-      <c r="K74" s="12" t="n"/>
-      <c r="L74" s="17">
+      <c r="A74" s="11" t="n"/>
+      <c r="B74" s="11" t="n"/>
+      <c r="C74" s="11" t="n"/>
+      <c r="D74" s="11" t="n"/>
+      <c r="E74" s="11" t="n"/>
+      <c r="F74" s="11" t="n"/>
+      <c r="G74" s="11" t="n"/>
+      <c r="H74" s="12" t="n"/>
+      <c r="I74" s="12" t="n"/>
+      <c r="J74" s="11" t="n"/>
+      <c r="K74" s="11" t="n"/>
+      <c r="L74" s="13">
         <f>IF(A74="","",DAYS(TODAY(),J74))</f>
         <v/>
       </c>
-      <c r="M74" s="12" t="n"/>
+      <c r="M74" s="11" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="8" t="n"/>
@@ -3208,33 +2876,33 @@
       <c r="E75" s="8" t="n"/>
       <c r="F75" s="8" t="n"/>
       <c r="G75" s="8" t="n"/>
-      <c r="H75" s="18" t="n"/>
-      <c r="I75" s="18" t="n"/>
+      <c r="H75" s="9" t="n"/>
+      <c r="I75" s="9" t="n"/>
       <c r="J75" s="8" t="n"/>
       <c r="K75" s="8" t="n"/>
-      <c r="L75" s="19">
+      <c r="L75" s="10">
         <f>IF(A75="","",DAYS(TODAY(),J75))</f>
         <v/>
       </c>
       <c r="M75" s="8" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="12" t="n"/>
-      <c r="B76" s="12" t="n"/>
-      <c r="C76" s="12" t="n"/>
-      <c r="D76" s="12" t="n"/>
-      <c r="E76" s="12" t="n"/>
-      <c r="F76" s="12" t="n"/>
-      <c r="G76" s="12" t="n"/>
-      <c r="H76" s="16" t="n"/>
-      <c r="I76" s="16" t="n"/>
-      <c r="J76" s="12" t="n"/>
-      <c r="K76" s="12" t="n"/>
-      <c r="L76" s="17">
+      <c r="A76" s="11" t="n"/>
+      <c r="B76" s="11" t="n"/>
+      <c r="C76" s="11" t="n"/>
+      <c r="D76" s="11" t="n"/>
+      <c r="E76" s="11" t="n"/>
+      <c r="F76" s="11" t="n"/>
+      <c r="G76" s="11" t="n"/>
+      <c r="H76" s="12" t="n"/>
+      <c r="I76" s="12" t="n"/>
+      <c r="J76" s="11" t="n"/>
+      <c r="K76" s="11" t="n"/>
+      <c r="L76" s="13">
         <f>IF(A76="","",DAYS(TODAY(),J76))</f>
         <v/>
       </c>
-      <c r="M76" s="12" t="n"/>
+      <c r="M76" s="11" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="8" t="n"/>
@@ -3244,33 +2912,33 @@
       <c r="E77" s="8" t="n"/>
       <c r="F77" s="8" t="n"/>
       <c r="G77" s="8" t="n"/>
-      <c r="H77" s="18" t="n"/>
-      <c r="I77" s="18" t="n"/>
+      <c r="H77" s="9" t="n"/>
+      <c r="I77" s="9" t="n"/>
       <c r="J77" s="8" t="n"/>
       <c r="K77" s="8" t="n"/>
-      <c r="L77" s="19">
+      <c r="L77" s="10">
         <f>IF(A77="","",DAYS(TODAY(),J77))</f>
         <v/>
       </c>
       <c r="M77" s="8" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="12" t="n"/>
-      <c r="B78" s="12" t="n"/>
-      <c r="C78" s="12" t="n"/>
-      <c r="D78" s="12" t="n"/>
-      <c r="E78" s="12" t="n"/>
-      <c r="F78" s="12" t="n"/>
-      <c r="G78" s="12" t="n"/>
-      <c r="H78" s="16" t="n"/>
-      <c r="I78" s="16" t="n"/>
-      <c r="J78" s="12" t="n"/>
-      <c r="K78" s="12" t="n"/>
-      <c r="L78" s="17">
+      <c r="A78" s="11" t="n"/>
+      <c r="B78" s="11" t="n"/>
+      <c r="C78" s="11" t="n"/>
+      <c r="D78" s="11" t="n"/>
+      <c r="E78" s="11" t="n"/>
+      <c r="F78" s="11" t="n"/>
+      <c r="G78" s="11" t="n"/>
+      <c r="H78" s="12" t="n"/>
+      <c r="I78" s="12" t="n"/>
+      <c r="J78" s="11" t="n"/>
+      <c r="K78" s="11" t="n"/>
+      <c r="L78" s="13">
         <f>IF(A78="","",DAYS(TODAY(),J78))</f>
         <v/>
       </c>
-      <c r="M78" s="12" t="n"/>
+      <c r="M78" s="11" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="8" t="n"/>
@@ -3280,11 +2948,11 @@
       <c r="E79" s="8" t="n"/>
       <c r="F79" s="8" t="n"/>
       <c r="G79" s="8" t="n"/>
-      <c r="H79" s="18" t="n"/>
-      <c r="I79" s="18" t="n"/>
+      <c r="H79" s="9" t="n"/>
+      <c r="I79" s="9" t="n"/>
       <c r="J79" s="8" t="n"/>
       <c r="K79" s="8" t="n"/>
-      <c r="L79" s="19">
+      <c r="L79" s="10">
         <f>IF(A79="","",DAYS(TODAY(),J79))</f>
         <v/>
       </c>
@@ -3376,7 +3044,7 @@
   <sheetPr>
     <tabColor rgb="000F1B2D"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3399,67 +3067,67 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>TOTAL PIPELINE</t>
         </is>
       </c>
-      <c r="C3" s="20" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>EST. REVENUE</t>
         </is>
       </c>
-      <c r="E3" s="20" t="inlineStr">
+      <c r="E3" s="14" t="inlineStr">
         <is>
           <t>WON REVENUE</t>
         </is>
       </c>
-      <c r="G3" s="20" t="inlineStr">
+      <c r="G3" s="14" t="inlineStr">
         <is>
           <t>WIN RATE</t>
         </is>
       </c>
     </row>
     <row r="4" ht="50" customHeight="1">
-      <c r="A4" s="21">
+      <c r="A4" s="15">
         <f>SUMPRODUCT((Pipeline!F5:F80&lt;&gt;"Closed-Won")*(Pipeline!F5:F80&lt;&gt;"Closed-Lost")*(Pipeline!F5:F80&lt;&gt;"")*Pipeline!H5:H80)</f>
         <v/>
       </c>
-      <c r="C4" s="22">
+      <c r="C4" s="16">
         <f>SUMPRODUCT((Pipeline!F5:F80&lt;&gt;"Closed-Won")*(Pipeline!F5:F80&lt;&gt;"Closed-Lost")*(Pipeline!F5:F80&lt;&gt;"")*Pipeline!I5:I80)</f>
         <v/>
       </c>
-      <c r="E4" s="23">
+      <c r="E4" s="17">
         <f>SUMIF(Pipeline!F5:F80,"Closed-Won",Pipeline!I5:I80)</f>
         <v/>
       </c>
-      <c r="G4" s="24">
+      <c r="G4" s="18">
         <f>IFERROR(COUNTIF(Pipeline!F5:F80,"Closed-Won")/(COUNTIF(Pipeline!F5:F80,"Closed-Won")+COUNTIF(Pipeline!F5:F80,"Closed-Lost")),0)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="n"/>
-      <c r="B5" s="25" t="n"/>
-      <c r="C5" s="26" t="n"/>
-      <c r="D5" s="26" t="n"/>
-      <c r="E5" s="27" t="n"/>
-      <c r="F5" s="27" t="n"/>
-      <c r="G5" s="28" t="n"/>
-      <c r="H5" s="28" t="n"/>
+      <c r="A5" s="19" t="n"/>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="20" t="n"/>
+      <c r="D5" s="20" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="21" t="n"/>
+      <c r="G5" s="22" t="n"/>
+      <c r="H5" s="22" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="B20" s="29" t="inlineStr">
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C20" s="29" t="inlineStr">
+      <c r="C20" s="23" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
@@ -3475,7 +3143,7 @@
         <f>COUNTIF(Pipeline!F5:F80,A21)</f>
         <v/>
       </c>
-      <c r="C21" s="30">
+      <c r="C21" s="24">
         <f>SUMIF(Pipeline!F5:F80,A21,Pipeline!I5:I80)</f>
         <v/>
       </c>
@@ -3490,7 +3158,7 @@
         <f>COUNTIF(Pipeline!F5:F80,A22)</f>
         <v/>
       </c>
-      <c r="C22" s="30">
+      <c r="C22" s="24">
         <f>SUMIF(Pipeline!F5:F80,A22,Pipeline!I5:I80)</f>
         <v/>
       </c>
@@ -3505,7 +3173,7 @@
         <f>COUNTIF(Pipeline!F5:F80,A23)</f>
         <v/>
       </c>
-      <c r="C23" s="30">
+      <c r="C23" s="24">
         <f>SUMIF(Pipeline!F5:F80,A23,Pipeline!I5:I80)</f>
         <v/>
       </c>
@@ -3520,7 +3188,7 @@
         <f>COUNTIF(Pipeline!F5:F80,A24)</f>
         <v/>
       </c>
-      <c r="C24" s="30">
+      <c r="C24" s="24">
         <f>SUMIF(Pipeline!F5:F80,A24,Pipeline!I5:I80)</f>
         <v/>
       </c>
@@ -3535,7 +3203,7 @@
         <f>COUNTIF(Pipeline!F5:F80,A25)</f>
         <v/>
       </c>
-      <c r="C25" s="30">
+      <c r="C25" s="24">
         <f>SUMIF(Pipeline!F5:F80,A25,Pipeline!I5:I80)</f>
         <v/>
       </c>
@@ -3550,7 +3218,7 @@
         <f>COUNTIF(Pipeline!F5:F80,A26)</f>
         <v/>
       </c>
-      <c r="C26" s="30">
+      <c r="C26" s="24">
         <f>SUMIF(Pipeline!F5:F80,A26,Pipeline!I5:I80)</f>
         <v/>
       </c>
@@ -3565,7 +3233,7 @@
         <f>COUNTIF(Pipeline!F5:F80,A27)</f>
         <v/>
       </c>
-      <c r="C27" s="30">
+      <c r="C27" s="24">
         <f>SUMIF(Pipeline!F5:F80,A27,Pipeline!I5:I80)</f>
         <v/>
       </c>
@@ -3580,7 +3248,7 @@
         <f>COUNTIF(Pipeline!F5:F80,A28)</f>
         <v/>
       </c>
-      <c r="C28" s="30">
+      <c r="C28" s="24">
         <f>SUMIF(Pipeline!F5:F80,A28,Pipeline!I5:I80)</f>
         <v/>
       </c>
@@ -3595,7 +3263,7 @@
         <f>COUNTIF(Pipeline!F5:F80,A29)</f>
         <v/>
       </c>
-      <c r="C29" s="30">
+      <c r="C29" s="24">
         <f>SUMIF(Pipeline!F5:F80,A29,Pipeline!I5:I80)</f>
         <v/>
       </c>
@@ -3610,18 +3278,18 @@
         <f>COUNTIF(Pipeline!F5:F80,A30)</f>
         <v/>
       </c>
-      <c r="C30" s="30">
+      <c r="C30" s="24">
         <f>SUMIF(Pipeline!F5:F80,A30,Pipeline!I5:I80)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="29" t="inlineStr">
+      <c r="A33" s="23" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B33" s="29" t="inlineStr">
+      <c r="B33" s="23" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
@@ -3661,47 +3329,47 @@
       </c>
     </row>
     <row r="37" ht="32" customHeight="1">
-      <c r="A37" s="31" t="inlineStr">
+      <c r="A37" s="25" t="inlineStr">
         <is>
           <t>FOLLOW-UP STATUS</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="32" t="inlineStr">
+      <c r="A38" s="26" t="inlineStr">
         <is>
           <t>Overdue Follow-Ups</t>
         </is>
       </c>
-      <c r="B38" s="33" t="n"/>
-      <c r="C38" s="34" t="n"/>
-      <c r="D38" s="35">
+      <c r="B38" s="27" t="n"/>
+      <c r="C38" s="28" t="n"/>
+      <c r="D38" s="29">
         <f>COUNTIFS(Pipeline!K5:K80,"&lt;"&amp;TODAY(),Pipeline!K5:K80,"&lt;&gt;",Pipeline!F5:F80,"&lt;&gt;Closed-Won",Pipeline!F5:F80,"&lt;&gt;Closed-Lost")</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="32" t="inlineStr">
+      <c r="A39" s="26" t="inlineStr">
         <is>
           <t>Due Today</t>
         </is>
       </c>
-      <c r="B39" s="33" t="n"/>
-      <c r="C39" s="34" t="n"/>
-      <c r="D39" s="35">
+      <c r="B39" s="27" t="n"/>
+      <c r="C39" s="28" t="n"/>
+      <c r="D39" s="29">
         <f>COUNTIFS(Pipeline!K5:K80,TODAY(),Pipeline!F5:F80,"&lt;&gt;Closed-Won")</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="32" t="inlineStr">
+      <c r="A40" s="26" t="inlineStr">
         <is>
           <t>Due This Week</t>
         </is>
       </c>
-      <c r="B40" s="33" t="n"/>
-      <c r="C40" s="34" t="n"/>
-      <c r="D40" s="35">
+      <c r="B40" s="27" t="n"/>
+      <c r="C40" s="28" t="n"/>
+      <c r="D40" s="29">
         <f>COUNTIFS(Pipeline!K5:K80,"&gt;="&amp;TODAY(),Pipeline!K5:K80,"&lt;="&amp;(TODAY()+7),Pipeline!F5:F80,"&lt;&gt;Closed-Won")</f>
         <v/>
       </c>
@@ -3729,17 +3397,17 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="29" t="inlineStr">
+      <c r="A45" s="23" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="B45" s="29" t="inlineStr">
+      <c r="B45" s="23" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C45" s="29" t="inlineStr">
+      <c r="C45" s="23" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
@@ -3862,7 +3530,7 @@
   <sheetPr>
     <tabColor rgb="0027AE60"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3915,132 +3583,36 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>2026-03-08</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Priya Patel</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Video call - final proposal</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>Reviewing with spouse</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>Follow up Monday</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>Key person insurance quote included</t>
-        </is>
-      </c>
+      <c r="A3" s="8" t="n"/>
+      <c r="B3" s="8" t="n"/>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Jessica Williams</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>Presented full plan</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Loved it, wants to proceed</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Send engagement letter</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="inlineStr">
-        <is>
-          <t>Adding $1M term life to plan</t>
-        </is>
-      </c>
+      <c r="A4" s="11" t="n"/>
+      <c r="B4" s="11" t="n"/>
+      <c r="C4" s="11" t="n"/>
+      <c r="D4" s="11" t="n"/>
+      <c r="E4" s="11" t="n"/>
+      <c r="F4" s="11" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>Sarah Johnson</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Discovery call - 45 min</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>Good fit, moving forward</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>Send needs analysis</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>Needs $500K term + RESP + RRSP</t>
-        </is>
-      </c>
+      <c r="A5" s="8" t="n"/>
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>David Chen</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>Sent intro email</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Downloaded guide</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>Call next week</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>From website lead</t>
-        </is>
-      </c>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="11" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="n"/>
@@ -4051,12 +3623,12 @@
       <c r="F7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n"/>
-      <c r="B8" s="12" t="n"/>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="12" t="n"/>
-      <c r="E8" s="12" t="n"/>
-      <c r="F8" s="12" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n"/>
@@ -4067,12 +3639,12 @@
       <c r="F9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="12" t="n"/>
-      <c r="C10" s="12" t="n"/>
-      <c r="D10" s="12" t="n"/>
-      <c r="E10" s="12" t="n"/>
-      <c r="F10" s="12" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n"/>
@@ -4083,12 +3655,12 @@
       <c r="F11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="12" t="n"/>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="12" t="n"/>
-      <c r="F12" s="12" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n"/>
@@ -4099,12 +3671,12 @@
       <c r="F13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="12" t="n"/>
-      <c r="F14" s="12" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n"/>
@@ -4115,12 +3687,12 @@
       <c r="F15" s="8" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="12" t="n"/>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="12" t="n"/>
-      <c r="F16" s="12" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n"/>
@@ -4131,12 +3703,12 @@
       <c r="F17" s="8" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="12" t="n"/>
-      <c r="E18" s="12" t="n"/>
-      <c r="F18" s="12" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n"/>
@@ -4147,12 +3719,12 @@
       <c r="F19" s="8" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="12" t="n"/>
-      <c r="F20" s="12" t="n"/>
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n"/>
@@ -4163,12 +3735,12 @@
       <c r="F21" s="8" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="n"/>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="12" t="n"/>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="12" t="n"/>
-      <c r="F22" s="12" t="n"/>
+      <c r="A22" s="11" t="n"/>
+      <c r="B22" s="11" t="n"/>
+      <c r="C22" s="11" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="n"/>
@@ -4179,12 +3751,12 @@
       <c r="F23" s="8" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n"/>
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="12" t="n"/>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="12" t="n"/>
-      <c r="F24" s="12" t="n"/>
+      <c r="A24" s="11" t="n"/>
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="11" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n"/>
@@ -4195,12 +3767,12 @@
       <c r="F25" s="8" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="n"/>
-      <c r="B26" s="12" t="n"/>
-      <c r="C26" s="12" t="n"/>
-      <c r="D26" s="12" t="n"/>
-      <c r="E26" s="12" t="n"/>
-      <c r="F26" s="12" t="n"/>
+      <c r="A26" s="11" t="n"/>
+      <c r="B26" s="11" t="n"/>
+      <c r="C26" s="11" t="n"/>
+      <c r="D26" s="11" t="n"/>
+      <c r="E26" s="11" t="n"/>
+      <c r="F26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="n"/>
@@ -4211,12 +3783,12 @@
       <c r="F27" s="8" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n"/>
-      <c r="B28" s="12" t="n"/>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="12" t="n"/>
-      <c r="E28" s="12" t="n"/>
-      <c r="F28" s="12" t="n"/>
+      <c r="A28" s="11" t="n"/>
+      <c r="B28" s="11" t="n"/>
+      <c r="C28" s="11" t="n"/>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="n"/>
@@ -4227,12 +3799,12 @@
       <c r="F29" s="8" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n"/>
-      <c r="B30" s="12" t="n"/>
-      <c r="C30" s="12" t="n"/>
-      <c r="D30" s="12" t="n"/>
-      <c r="E30" s="12" t="n"/>
-      <c r="F30" s="12" t="n"/>
+      <c r="A30" s="11" t="n"/>
+      <c r="B30" s="11" t="n"/>
+      <c r="C30" s="11" t="n"/>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="n"/>
@@ -4243,12 +3815,12 @@
       <c r="F31" s="8" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="n"/>
-      <c r="B32" s="12" t="n"/>
-      <c r="C32" s="12" t="n"/>
-      <c r="D32" s="12" t="n"/>
-      <c r="E32" s="12" t="n"/>
-      <c r="F32" s="12" t="n"/>
+      <c r="A32" s="11" t="n"/>
+      <c r="B32" s="11" t="n"/>
+      <c r="C32" s="11" t="n"/>
+      <c r="D32" s="11" t="n"/>
+      <c r="E32" s="11" t="n"/>
+      <c r="F32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="n"/>
@@ -4259,12 +3831,12 @@
       <c r="F33" s="8" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="n"/>
-      <c r="B34" s="12" t="n"/>
-      <c r="C34" s="12" t="n"/>
-      <c r="D34" s="12" t="n"/>
-      <c r="E34" s="12" t="n"/>
-      <c r="F34" s="12" t="n"/>
+      <c r="A34" s="11" t="n"/>
+      <c r="B34" s="11" t="n"/>
+      <c r="C34" s="11" t="n"/>
+      <c r="D34" s="11" t="n"/>
+      <c r="E34" s="11" t="n"/>
+      <c r="F34" s="11" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="8" t="n"/>
@@ -4275,12 +3847,12 @@
       <c r="F35" s="8" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="n"/>
-      <c r="B36" s="12" t="n"/>
-      <c r="C36" s="12" t="n"/>
-      <c r="D36" s="12" t="n"/>
-      <c r="E36" s="12" t="n"/>
-      <c r="F36" s="12" t="n"/>
+      <c r="A36" s="11" t="n"/>
+      <c r="B36" s="11" t="n"/>
+      <c r="C36" s="11" t="n"/>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="11" t="n"/>
+      <c r="F36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="n"/>
@@ -4291,12 +3863,12 @@
       <c r="F37" s="8" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="12" t="n"/>
-      <c r="B38" s="12" t="n"/>
-      <c r="C38" s="12" t="n"/>
-      <c r="D38" s="12" t="n"/>
-      <c r="E38" s="12" t="n"/>
-      <c r="F38" s="12" t="n"/>
+      <c r="A38" s="11" t="n"/>
+      <c r="B38" s="11" t="n"/>
+      <c r="C38" s="11" t="n"/>
+      <c r="D38" s="11" t="n"/>
+      <c r="E38" s="11" t="n"/>
+      <c r="F38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="n"/>
@@ -4307,12 +3879,12 @@
       <c r="F39" s="8" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="12" t="n"/>
-      <c r="B40" s="12" t="n"/>
-      <c r="C40" s="12" t="n"/>
-      <c r="D40" s="12" t="n"/>
-      <c r="E40" s="12" t="n"/>
-      <c r="F40" s="12" t="n"/>
+      <c r="A40" s="11" t="n"/>
+      <c r="B40" s="11" t="n"/>
+      <c r="C40" s="11" t="n"/>
+      <c r="D40" s="11" t="n"/>
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="8" t="n"/>
@@ -4323,12 +3895,12 @@
       <c r="F41" s="8" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="12" t="n"/>
-      <c r="B42" s="12" t="n"/>
-      <c r="C42" s="12" t="n"/>
-      <c r="D42" s="12" t="n"/>
-      <c r="E42" s="12" t="n"/>
-      <c r="F42" s="12" t="n"/>
+      <c r="A42" s="11" t="n"/>
+      <c r="B42" s="11" t="n"/>
+      <c r="C42" s="11" t="n"/>
+      <c r="D42" s="11" t="n"/>
+      <c r="E42" s="11" t="n"/>
+      <c r="F42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="8" t="n"/>
@@ -4339,12 +3911,12 @@
       <c r="F43" s="8" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="n"/>
-      <c r="B44" s="12" t="n"/>
-      <c r="C44" s="12" t="n"/>
-      <c r="D44" s="12" t="n"/>
-      <c r="E44" s="12" t="n"/>
-      <c r="F44" s="12" t="n"/>
+      <c r="A44" s="11" t="n"/>
+      <c r="B44" s="11" t="n"/>
+      <c r="C44" s="11" t="n"/>
+      <c r="D44" s="11" t="n"/>
+      <c r="E44" s="11" t="n"/>
+      <c r="F44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="n"/>
@@ -4355,12 +3927,12 @@
       <c r="F45" s="8" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="12" t="n"/>
-      <c r="B46" s="12" t="n"/>
-      <c r="C46" s="12" t="n"/>
-      <c r="D46" s="12" t="n"/>
-      <c r="E46" s="12" t="n"/>
-      <c r="F46" s="12" t="n"/>
+      <c r="A46" s="11" t="n"/>
+      <c r="B46" s="11" t="n"/>
+      <c r="C46" s="11" t="n"/>
+      <c r="D46" s="11" t="n"/>
+      <c r="E46" s="11" t="n"/>
+      <c r="F46" s="11" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="8" t="n"/>
@@ -4371,12 +3943,12 @@
       <c r="F47" s="8" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="12" t="n"/>
-      <c r="B48" s="12" t="n"/>
-      <c r="C48" s="12" t="n"/>
-      <c r="D48" s="12" t="n"/>
-      <c r="E48" s="12" t="n"/>
-      <c r="F48" s="12" t="n"/>
+      <c r="A48" s="11" t="n"/>
+      <c r="B48" s="11" t="n"/>
+      <c r="C48" s="11" t="n"/>
+      <c r="D48" s="11" t="n"/>
+      <c r="E48" s="11" t="n"/>
+      <c r="F48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="8" t="n"/>
@@ -4387,12 +3959,12 @@
       <c r="F49" s="8" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="12" t="n"/>
-      <c r="B50" s="12" t="n"/>
-      <c r="C50" s="12" t="n"/>
-      <c r="D50" s="12" t="n"/>
-      <c r="E50" s="12" t="n"/>
-      <c r="F50" s="12" t="n"/>
+      <c r="A50" s="11" t="n"/>
+      <c r="B50" s="11" t="n"/>
+      <c r="C50" s="11" t="n"/>
+      <c r="D50" s="11" t="n"/>
+      <c r="E50" s="11" t="n"/>
+      <c r="F50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="n"/>
@@ -4403,12 +3975,12 @@
       <c r="F51" s="8" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="12" t="n"/>
-      <c r="B52" s="12" t="n"/>
-      <c r="C52" s="12" t="n"/>
-      <c r="D52" s="12" t="n"/>
-      <c r="E52" s="12" t="n"/>
-      <c r="F52" s="12" t="n"/>
+      <c r="A52" s="11" t="n"/>
+      <c r="B52" s="11" t="n"/>
+      <c r="C52" s="11" t="n"/>
+      <c r="D52" s="11" t="n"/>
+      <c r="E52" s="11" t="n"/>
+      <c r="F52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="8" t="n"/>
@@ -4419,12 +3991,12 @@
       <c r="F53" s="8" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="12" t="n"/>
-      <c r="B54" s="12" t="n"/>
-      <c r="C54" s="12" t="n"/>
-      <c r="D54" s="12" t="n"/>
-      <c r="E54" s="12" t="n"/>
-      <c r="F54" s="12" t="n"/>
+      <c r="A54" s="11" t="n"/>
+      <c r="B54" s="11" t="n"/>
+      <c r="C54" s="11" t="n"/>
+      <c r="D54" s="11" t="n"/>
+      <c r="E54" s="11" t="n"/>
+      <c r="F54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="8" t="n"/>
@@ -4435,12 +4007,12 @@
       <c r="F55" s="8" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="12" t="n"/>
-      <c r="B56" s="12" t="n"/>
-      <c r="C56" s="12" t="n"/>
-      <c r="D56" s="12" t="n"/>
-      <c r="E56" s="12" t="n"/>
-      <c r="F56" s="12" t="n"/>
+      <c r="A56" s="11" t="n"/>
+      <c r="B56" s="11" t="n"/>
+      <c r="C56" s="11" t="n"/>
+      <c r="D56" s="11" t="n"/>
+      <c r="E56" s="11" t="n"/>
+      <c r="F56" s="11" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="8" t="n"/>
@@ -4451,12 +4023,12 @@
       <c r="F57" s="8" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="12" t="n"/>
-      <c r="B58" s="12" t="n"/>
-      <c r="C58" s="12" t="n"/>
-      <c r="D58" s="12" t="n"/>
-      <c r="E58" s="12" t="n"/>
-      <c r="F58" s="12" t="n"/>
+      <c r="A58" s="11" t="n"/>
+      <c r="B58" s="11" t="n"/>
+      <c r="C58" s="11" t="n"/>
+      <c r="D58" s="11" t="n"/>
+      <c r="E58" s="11" t="n"/>
+      <c r="F58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n"/>
@@ -4467,12 +4039,12 @@
       <c r="F59" s="8" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="12" t="n"/>
-      <c r="B60" s="12" t="n"/>
-      <c r="C60" s="12" t="n"/>
-      <c r="D60" s="12" t="n"/>
-      <c r="E60" s="12" t="n"/>
-      <c r="F60" s="12" t="n"/>
+      <c r="A60" s="11" t="n"/>
+      <c r="B60" s="11" t="n"/>
+      <c r="C60" s="11" t="n"/>
+      <c r="D60" s="11" t="n"/>
+      <c r="E60" s="11" t="n"/>
+      <c r="F60" s="11" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="8" t="n"/>
@@ -4483,12 +4055,12 @@
       <c r="F61" s="8" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="12" t="n"/>
-      <c r="B62" s="12" t="n"/>
-      <c r="C62" s="12" t="n"/>
-      <c r="D62" s="12" t="n"/>
-      <c r="E62" s="12" t="n"/>
-      <c r="F62" s="12" t="n"/>
+      <c r="A62" s="11" t="n"/>
+      <c r="B62" s="11" t="n"/>
+      <c r="C62" s="11" t="n"/>
+      <c r="D62" s="11" t="n"/>
+      <c r="E62" s="11" t="n"/>
+      <c r="F62" s="11" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="8" t="n"/>
@@ -4499,12 +4071,12 @@
       <c r="F63" s="8" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="12" t="n"/>
-      <c r="B64" s="12" t="n"/>
-      <c r="C64" s="12" t="n"/>
-      <c r="D64" s="12" t="n"/>
-      <c r="E64" s="12" t="n"/>
-      <c r="F64" s="12" t="n"/>
+      <c r="A64" s="11" t="n"/>
+      <c r="B64" s="11" t="n"/>
+      <c r="C64" s="11" t="n"/>
+      <c r="D64" s="11" t="n"/>
+      <c r="E64" s="11" t="n"/>
+      <c r="F64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="8" t="n"/>
@@ -4515,12 +4087,12 @@
       <c r="F65" s="8" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="12" t="n"/>
-      <c r="B66" s="12" t="n"/>
-      <c r="C66" s="12" t="n"/>
-      <c r="D66" s="12" t="n"/>
-      <c r="E66" s="12" t="n"/>
-      <c r="F66" s="12" t="n"/>
+      <c r="A66" s="11" t="n"/>
+      <c r="B66" s="11" t="n"/>
+      <c r="C66" s="11" t="n"/>
+      <c r="D66" s="11" t="n"/>
+      <c r="E66" s="11" t="n"/>
+      <c r="F66" s="11" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="8" t="n"/>
@@ -4531,12 +4103,12 @@
       <c r="F67" s="8" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="12" t="n"/>
-      <c r="B68" s="12" t="n"/>
-      <c r="C68" s="12" t="n"/>
-      <c r="D68" s="12" t="n"/>
-      <c r="E68" s="12" t="n"/>
-      <c r="F68" s="12" t="n"/>
+      <c r="A68" s="11" t="n"/>
+      <c r="B68" s="11" t="n"/>
+      <c r="C68" s="11" t="n"/>
+      <c r="D68" s="11" t="n"/>
+      <c r="E68" s="11" t="n"/>
+      <c r="F68" s="11" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="8" t="n"/>
@@ -4547,12 +4119,12 @@
       <c r="F69" s="8" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="12" t="n"/>
-      <c r="B70" s="12" t="n"/>
-      <c r="C70" s="12" t="n"/>
-      <c r="D70" s="12" t="n"/>
-      <c r="E70" s="12" t="n"/>
-      <c r="F70" s="12" t="n"/>
+      <c r="A70" s="11" t="n"/>
+      <c r="B70" s="11" t="n"/>
+      <c r="C70" s="11" t="n"/>
+      <c r="D70" s="11" t="n"/>
+      <c r="E70" s="11" t="n"/>
+      <c r="F70" s="11" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="8" t="n"/>
@@ -4563,12 +4135,12 @@
       <c r="F71" s="8" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="12" t="n"/>
-      <c r="B72" s="12" t="n"/>
-      <c r="C72" s="12" t="n"/>
-      <c r="D72" s="12" t="n"/>
-      <c r="E72" s="12" t="n"/>
-      <c r="F72" s="12" t="n"/>
+      <c r="A72" s="11" t="n"/>
+      <c r="B72" s="11" t="n"/>
+      <c r="C72" s="11" t="n"/>
+      <c r="D72" s="11" t="n"/>
+      <c r="E72" s="11" t="n"/>
+      <c r="F72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="8" t="n"/>
@@ -4579,12 +4151,12 @@
       <c r="F73" s="8" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="12" t="n"/>
-      <c r="B74" s="12" t="n"/>
-      <c r="C74" s="12" t="n"/>
-      <c r="D74" s="12" t="n"/>
-      <c r="E74" s="12" t="n"/>
-      <c r="F74" s="12" t="n"/>
+      <c r="A74" s="11" t="n"/>
+      <c r="B74" s="11" t="n"/>
+      <c r="C74" s="11" t="n"/>
+      <c r="D74" s="11" t="n"/>
+      <c r="E74" s="11" t="n"/>
+      <c r="F74" s="11" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="8" t="n"/>
@@ -4595,12 +4167,12 @@
       <c r="F75" s="8" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="12" t="n"/>
-      <c r="B76" s="12" t="n"/>
-      <c r="C76" s="12" t="n"/>
-      <c r="D76" s="12" t="n"/>
-      <c r="E76" s="12" t="n"/>
-      <c r="F76" s="12" t="n"/>
+      <c r="A76" s="11" t="n"/>
+      <c r="B76" s="11" t="n"/>
+      <c r="C76" s="11" t="n"/>
+      <c r="D76" s="11" t="n"/>
+      <c r="E76" s="11" t="n"/>
+      <c r="F76" s="11" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="8" t="n"/>
@@ -4611,12 +4183,12 @@
       <c r="F77" s="8" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="12" t="n"/>
-      <c r="B78" s="12" t="n"/>
-      <c r="C78" s="12" t="n"/>
-      <c r="D78" s="12" t="n"/>
-      <c r="E78" s="12" t="n"/>
-      <c r="F78" s="12" t="n"/>
+      <c r="A78" s="11" t="n"/>
+      <c r="B78" s="11" t="n"/>
+      <c r="C78" s="11" t="n"/>
+      <c r="D78" s="11" t="n"/>
+      <c r="E78" s="11" t="n"/>
+      <c r="F78" s="11" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="8" t="n"/>
@@ -4627,12 +4199,12 @@
       <c r="F79" s="8" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="12" t="n"/>
-      <c r="B80" s="12" t="n"/>
-      <c r="C80" s="12" t="n"/>
-      <c r="D80" s="12" t="n"/>
-      <c r="E80" s="12" t="n"/>
-      <c r="F80" s="12" t="n"/>
+      <c r="A80" s="11" t="n"/>
+      <c r="B80" s="11" t="n"/>
+      <c r="C80" s="11" t="n"/>
+      <c r="D80" s="11" t="n"/>
+      <c r="E80" s="11" t="n"/>
+      <c r="F80" s="11" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="8" t="n"/>
@@ -4643,12 +4215,12 @@
       <c r="F81" s="8" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="12" t="n"/>
-      <c r="B82" s="12" t="n"/>
-      <c r="C82" s="12" t="n"/>
-      <c r="D82" s="12" t="n"/>
-      <c r="E82" s="12" t="n"/>
-      <c r="F82" s="12" t="n"/>
+      <c r="A82" s="11" t="n"/>
+      <c r="B82" s="11" t="n"/>
+      <c r="C82" s="11" t="n"/>
+      <c r="D82" s="11" t="n"/>
+      <c r="E82" s="11" t="n"/>
+      <c r="F82" s="11" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="8" t="n"/>
@@ -4659,12 +4231,12 @@
       <c r="F83" s="8" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="12" t="n"/>
-      <c r="B84" s="12" t="n"/>
-      <c r="C84" s="12" t="n"/>
-      <c r="D84" s="12" t="n"/>
-      <c r="E84" s="12" t="n"/>
-      <c r="F84" s="12" t="n"/>
+      <c r="A84" s="11" t="n"/>
+      <c r="B84" s="11" t="n"/>
+      <c r="C84" s="11" t="n"/>
+      <c r="D84" s="11" t="n"/>
+      <c r="E84" s="11" t="n"/>
+      <c r="F84" s="11" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="8" t="n"/>
@@ -4675,12 +4247,12 @@
       <c r="F85" s="8" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="12" t="n"/>
-      <c r="B86" s="12" t="n"/>
-      <c r="C86" s="12" t="n"/>
-      <c r="D86" s="12" t="n"/>
-      <c r="E86" s="12" t="n"/>
-      <c r="F86" s="12" t="n"/>
+      <c r="A86" s="11" t="n"/>
+      <c r="B86" s="11" t="n"/>
+      <c r="C86" s="11" t="n"/>
+      <c r="D86" s="11" t="n"/>
+      <c r="E86" s="11" t="n"/>
+      <c r="F86" s="11" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="8" t="n"/>
@@ -4691,12 +4263,12 @@
       <c r="F87" s="8" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="12" t="n"/>
-      <c r="B88" s="12" t="n"/>
-      <c r="C88" s="12" t="n"/>
-      <c r="D88" s="12" t="n"/>
-      <c r="E88" s="12" t="n"/>
-      <c r="F88" s="12" t="n"/>
+      <c r="A88" s="11" t="n"/>
+      <c r="B88" s="11" t="n"/>
+      <c r="C88" s="11" t="n"/>
+      <c r="D88" s="11" t="n"/>
+      <c r="E88" s="11" t="n"/>
+      <c r="F88" s="11" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="8" t="n"/>
@@ -4707,12 +4279,12 @@
       <c r="F89" s="8" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="12" t="n"/>
-      <c r="B90" s="12" t="n"/>
-      <c r="C90" s="12" t="n"/>
-      <c r="D90" s="12" t="n"/>
-      <c r="E90" s="12" t="n"/>
-      <c r="F90" s="12" t="n"/>
+      <c r="A90" s="11" t="n"/>
+      <c r="B90" s="11" t="n"/>
+      <c r="C90" s="11" t="n"/>
+      <c r="D90" s="11" t="n"/>
+      <c r="E90" s="11" t="n"/>
+      <c r="F90" s="11" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="8" t="n"/>
@@ -4723,12 +4295,12 @@
       <c r="F91" s="8" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="12" t="n"/>
-      <c r="B92" s="12" t="n"/>
-      <c r="C92" s="12" t="n"/>
-      <c r="D92" s="12" t="n"/>
-      <c r="E92" s="12" t="n"/>
-      <c r="F92" s="12" t="n"/>
+      <c r="A92" s="11" t="n"/>
+      <c r="B92" s="11" t="n"/>
+      <c r="C92" s="11" t="n"/>
+      <c r="D92" s="11" t="n"/>
+      <c r="E92" s="11" t="n"/>
+      <c r="F92" s="11" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="8" t="n"/>
@@ -4739,12 +4311,12 @@
       <c r="F93" s="8" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="12" t="n"/>
-      <c r="B94" s="12" t="n"/>
-      <c r="C94" s="12" t="n"/>
-      <c r="D94" s="12" t="n"/>
-      <c r="E94" s="12" t="n"/>
-      <c r="F94" s="12" t="n"/>
+      <c r="A94" s="11" t="n"/>
+      <c r="B94" s="11" t="n"/>
+      <c r="C94" s="11" t="n"/>
+      <c r="D94" s="11" t="n"/>
+      <c r="E94" s="11" t="n"/>
+      <c r="F94" s="11" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="8" t="n"/>
@@ -4755,12 +4327,12 @@
       <c r="F95" s="8" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="12" t="n"/>
-      <c r="B96" s="12" t="n"/>
-      <c r="C96" s="12" t="n"/>
-      <c r="D96" s="12" t="n"/>
-      <c r="E96" s="12" t="n"/>
-      <c r="F96" s="12" t="n"/>
+      <c r="A96" s="11" t="n"/>
+      <c r="B96" s="11" t="n"/>
+      <c r="C96" s="11" t="n"/>
+      <c r="D96" s="11" t="n"/>
+      <c r="E96" s="11" t="n"/>
+      <c r="F96" s="11" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="8" t="n"/>
@@ -4771,12 +4343,12 @@
       <c r="F97" s="8" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="12" t="n"/>
-      <c r="B98" s="12" t="n"/>
-      <c r="C98" s="12" t="n"/>
-      <c r="D98" s="12" t="n"/>
-      <c r="E98" s="12" t="n"/>
-      <c r="F98" s="12" t="n"/>
+      <c r="A98" s="11" t="n"/>
+      <c r="B98" s="11" t="n"/>
+      <c r="C98" s="11" t="n"/>
+      <c r="D98" s="11" t="n"/>
+      <c r="E98" s="11" t="n"/>
+      <c r="F98" s="11" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="8" t="n"/>
@@ -4787,12 +4359,12 @@
       <c r="F99" s="8" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="12" t="n"/>
-      <c r="B100" s="12" t="n"/>
-      <c r="C100" s="12" t="n"/>
-      <c r="D100" s="12" t="n"/>
-      <c r="E100" s="12" t="n"/>
-      <c r="F100" s="12" t="n"/>
+      <c r="A100" s="11" t="n"/>
+      <c r="B100" s="11" t="n"/>
+      <c r="C100" s="11" t="n"/>
+      <c r="D100" s="11" t="n"/>
+      <c r="E100" s="11" t="n"/>
+      <c r="F100" s="11" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="8" t="n"/>
@@ -4803,12 +4375,12 @@
       <c r="F101" s="8" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="12" t="n"/>
-      <c r="B102" s="12" t="n"/>
-      <c r="C102" s="12" t="n"/>
-      <c r="D102" s="12" t="n"/>
-      <c r="E102" s="12" t="n"/>
-      <c r="F102" s="12" t="n"/>
+      <c r="A102" s="11" t="n"/>
+      <c r="B102" s="11" t="n"/>
+      <c r="C102" s="11" t="n"/>
+      <c r="D102" s="11" t="n"/>
+      <c r="E102" s="11" t="n"/>
+      <c r="F102" s="11" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:F102"/>
@@ -4833,7 +4405,7 @@
   <sheetPr>
     <tabColor rgb="00F39C12"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4852,92 +4424,80 @@
       </c>
     </row>
     <row r="3" ht="32" customHeight="1">
-      <c r="A3" s="31" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>THIS WEEK'S NUMBERS</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="36" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>Active Deals</t>
         </is>
       </c>
-      <c r="B4" s="34" t="n"/>
-      <c r="C4" s="37">
+      <c r="C4" s="31">
         <f>COUNTIFS(Pipeline!A5:A80,"&lt;&gt;",Pipeline!F5:F80,"&lt;&gt;Closed-Won",Pipeline!F5:F80,"&lt;&gt;Closed-Lost")</f>
         <v/>
       </c>
-      <c r="D4" s="34" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="36" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>Pipeline Value</t>
         </is>
       </c>
-      <c r="B5" s="34" t="n"/>
-      <c r="C5" s="38">
+      <c r="C5" s="32">
         <f>SUMPRODUCT((Pipeline!F5:F80&lt;&gt;"Closed-Won")*(Pipeline!F5:F80&lt;&gt;"Closed-Lost")*(Pipeline!F5:F80&lt;&gt;"")*Pipeline!H5:H80)</f>
         <v/>
       </c>
-      <c r="D5" s="34" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>Hot Leads</t>
         </is>
       </c>
-      <c r="B6" s="34" t="n"/>
-      <c r="C6" s="37">
+      <c r="C6" s="31">
         <f>COUNTIF(Pipeline!E5:E80,"Hot")</f>
         <v/>
       </c>
-      <c r="D6" s="34" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="36" t="inlineStr">
+      <c r="A7" s="30" t="inlineStr">
         <is>
           <t>Overdue Follow-Ups</t>
         </is>
       </c>
-      <c r="B7" s="34" t="n"/>
-      <c r="C7" s="37">
+      <c r="C7" s="31">
         <f>COUNTIFS(Pipeline!K5:K80,"&lt;"&amp;TODAY(),Pipeline!K5:K80,"&lt;&gt;",Pipeline!F5:F80,"&lt;&gt;Closed-Won",Pipeline!F5:F80,"&lt;&gt;Closed-Lost")</f>
         <v/>
       </c>
-      <c r="D7" s="34" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="36" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>Follow-Ups This Week</t>
         </is>
       </c>
-      <c r="B8" s="34" t="n"/>
-      <c r="C8" s="37">
+      <c r="C8" s="31">
         <f>COUNTIFS(Pipeline!K5:K80,"&gt;="&amp;TODAY(),Pipeline!K5:K80,"&lt;="&amp;(TODAY()+7),Pipeline!F5:F80,"&lt;&gt;Closed-Won")</f>
         <v/>
       </c>
-      <c r="D8" s="34" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="36" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>Deals Won (Total)</t>
         </is>
       </c>
-      <c r="B9" s="34" t="n"/>
-      <c r="C9" s="37">
+      <c r="C9" s="31">
         <f>COUNTIF(Pipeline!F5:F80,"Closed-Won")</f>
         <v/>
       </c>
-      <c r="D9" s="34" t="n"/>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>TOP 5 ACTIONS THIS WEEK</t>
         </is>
@@ -4972,10 +4532,10 @@
       <c r="D13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="12" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n"/>
@@ -4984,10 +4544,10 @@
       <c r="D15" s="8" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="12" t="n"/>
-      <c r="D16" s="12" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n"/>
@@ -4996,66 +4556,48 @@
       <c r="D17" s="8" t="n"/>
     </row>
     <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="31" t="inlineStr">
+      <c r="A19" s="25" t="inlineStr">
         <is>
           <t>WINS THIS WEEK</t>
         </is>
       </c>
     </row>
     <row r="20" ht="25" customHeight="1">
-      <c r="A20" s="39" t="n"/>
-      <c r="B20" s="33" t="n"/>
-      <c r="C20" s="33" t="n"/>
-      <c r="D20" s="34" t="n"/>
+      <c r="A20" s="33" t="n"/>
     </row>
     <row r="21" ht="25" customHeight="1">
-      <c r="A21" s="40" t="n"/>
-      <c r="B21" s="33" t="n"/>
-      <c r="C21" s="33" t="n"/>
-      <c r="D21" s="34" t="n"/>
+      <c r="A21" s="34" t="n"/>
     </row>
     <row r="22" ht="25" customHeight="1">
-      <c r="A22" s="39" t="n"/>
-      <c r="B22" s="33" t="n"/>
-      <c r="C22" s="33" t="n"/>
-      <c r="D22" s="34" t="n"/>
+      <c r="A22" s="33" t="n"/>
     </row>
     <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="31" t="inlineStr">
+      <c r="A24" s="25" t="inlineStr">
         <is>
           <t>NEXT WEEK'S FOCUS</t>
         </is>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="32" t="inlineStr">
+      <c r="A25" s="26" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B25" s="33" t="n"/>
-      <c r="C25" s="33" t="n"/>
-      <c r="D25" s="34" t="n"/>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="32" t="inlineStr">
+      <c r="A26" s="26" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B26" s="33" t="n"/>
-      <c r="C26" s="33" t="n"/>
-      <c r="D26" s="34" t="n"/>
     </row>
     <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="32" t="inlineStr">
+      <c r="A27" s="26" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B27" s="33" t="n"/>
-      <c r="C27" s="33" t="n"/>
-      <c r="D27" s="34" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="23">

</xml_diff>

<commit_message>
Add term life and disability insurance quote tools
- Term life: Co-operators rates via COMPULIFE API (scrape_rates.py), 132 rates scraped so far (ages 20-21), resumable scraper
- Disability: Edge Benefits rates extracted from client-side rate engine (5,974 rates + 2,119 occupation mappings), covers all risk classes, benefit amounts, wait periods, and benefit periods
- Both tools integrated into bot with Claude tool-use pattern
- Disability quotes auto-calculate max eligible benefit from income and look up occupation risk class

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline.xlsx
+++ b/pipeline.xlsx
@@ -11,6 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Review" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meetings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insurance Book" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pipeline'!$A$4:$M$80</definedName>
@@ -552,7 +554,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -742,7 +743,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -826,7 +826,6 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -986,7 +985,6 @@
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -4436,10 +4434,12 @@
           <t>Active Deals</t>
         </is>
       </c>
+      <c r="B4" s="28" t="n"/>
       <c r="C4" s="31">
         <f>COUNTIFS(Pipeline!A5:A80,"&lt;&gt;",Pipeline!F5:F80,"&lt;&gt;Closed-Won",Pipeline!F5:F80,"&lt;&gt;Closed-Lost")</f>
         <v/>
       </c>
+      <c r="D4" s="28" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="30" t="inlineStr">
@@ -4447,10 +4447,12 @@
           <t>Pipeline Value</t>
         </is>
       </c>
+      <c r="B5" s="28" t="n"/>
       <c r="C5" s="32">
         <f>SUMPRODUCT((Pipeline!F5:F80&lt;&gt;"Closed-Won")*(Pipeline!F5:F80&lt;&gt;"Closed-Lost")*(Pipeline!F5:F80&lt;&gt;"")*Pipeline!H5:H80)</f>
         <v/>
       </c>
+      <c r="D5" s="28" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="30" t="inlineStr">
@@ -4458,10 +4460,12 @@
           <t>Hot Leads</t>
         </is>
       </c>
+      <c r="B6" s="28" t="n"/>
       <c r="C6" s="31">
         <f>COUNTIF(Pipeline!E5:E80,"Hot")</f>
         <v/>
       </c>
+      <c r="D6" s="28" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="30" t="inlineStr">
@@ -4469,10 +4473,12 @@
           <t>Overdue Follow-Ups</t>
         </is>
       </c>
+      <c r="B7" s="28" t="n"/>
       <c r="C7" s="31">
         <f>COUNTIFS(Pipeline!K5:K80,"&lt;"&amp;TODAY(),Pipeline!K5:K80,"&lt;&gt;",Pipeline!F5:F80,"&lt;&gt;Closed-Won",Pipeline!F5:F80,"&lt;&gt;Closed-Lost")</f>
         <v/>
       </c>
+      <c r="D7" s="28" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="30" t="inlineStr">
@@ -4480,10 +4486,12 @@
           <t>Follow-Ups This Week</t>
         </is>
       </c>
+      <c r="B8" s="28" t="n"/>
       <c r="C8" s="31">
         <f>COUNTIFS(Pipeline!K5:K80,"&gt;="&amp;TODAY(),Pipeline!K5:K80,"&lt;="&amp;(TODAY()+7),Pipeline!F5:F80,"&lt;&gt;Closed-Won")</f>
         <v/>
       </c>
+      <c r="D8" s="28" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="30" t="inlineStr">
@@ -4491,10 +4499,12 @@
           <t>Deals Won (Total)</t>
         </is>
       </c>
+      <c r="B9" s="28" t="n"/>
       <c r="C9" s="31">
         <f>COUNTIF(Pipeline!F5:F80,"Closed-Won")</f>
         <v/>
       </c>
+      <c r="D9" s="28" t="n"/>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
@@ -4564,12 +4574,21 @@
     </row>
     <row r="20" ht="25" customHeight="1">
       <c r="A20" s="33" t="n"/>
+      <c r="B20" s="27" t="n"/>
+      <c r="C20" s="27" t="n"/>
+      <c r="D20" s="28" t="n"/>
     </row>
     <row r="21" ht="25" customHeight="1">
       <c r="A21" s="34" t="n"/>
+      <c r="B21" s="27" t="n"/>
+      <c r="C21" s="27" t="n"/>
+      <c r="D21" s="28" t="n"/>
     </row>
     <row r="22" ht="25" customHeight="1">
       <c r="A22" s="33" t="n"/>
+      <c r="B22" s="27" t="n"/>
+      <c r="C22" s="27" t="n"/>
+      <c r="D22" s="28" t="n"/>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="25" t="inlineStr">
@@ -4584,6 +4603,9 @@
           <t>1.</t>
         </is>
       </c>
+      <c r="B25" s="27" t="n"/>
+      <c r="C25" s="27" t="n"/>
+      <c r="D25" s="28" t="n"/>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
@@ -4591,6 +4613,9 @@
           <t>2.</t>
         </is>
       </c>
+      <c r="B26" s="27" t="n"/>
+      <c r="C26" s="27" t="n"/>
+      <c r="D26" s="28" t="n"/>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
@@ -4598,6 +4623,9 @@
           <t>3.</t>
         </is>
       </c>
+      <c r="B27" s="27" t="n"/>
+      <c r="C27" s="27" t="n"/>
+      <c r="D27" s="28" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="23">
@@ -4638,4 +4666,144 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="50" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MEETINGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Prep Notes</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="50" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>INSURANCE BOOK</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Policy Start</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Last Called</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Retry Date</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: _parse_numeric returns 0 instead of None, add *.db to gitignore
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline.xlsx
+++ b/pipeline.xlsx
@@ -1607,52 +1607,112 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n"/>
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Justin Douglas</t>
+        </is>
+      </c>
       <c r="B5" s="8" t="n"/>
       <c r="C5" s="8" t="n"/>
       <c r="D5" s="8" t="n"/>
       <c r="E5" s="8" t="n"/>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Proposal Sent</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Life Insurance</t>
+        </is>
+      </c>
       <c r="H5" s="9" t="n"/>
-      <c r="I5" s="9" t="n"/>
-      <c r="J5" s="8" t="n"/>
-      <c r="K5" s="8" t="n"/>
+      <c r="I5" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
       <c r="L5" s="10">
         <f>IF(A5="","",DAYS(TODAY(),J5))</f>
         <v/>
       </c>
-      <c r="M5" s="8" t="n"/>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>needs PHQ</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="n"/>
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Justin Douglas</t>
+        </is>
+      </c>
       <c r="B6" s="11" t="n"/>
       <c r="C6" s="11" t="n"/>
       <c r="D6" s="11" t="n"/>
       <c r="E6" s="11" t="n"/>
-      <c r="F6" s="11" t="n"/>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
       <c r="G6" s="11" t="n"/>
       <c r="H6" s="12" t="n"/>
       <c r="I6" s="12" t="n"/>
-      <c r="J6" s="11" t="n"/>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K6" s="11" t="n"/>
       <c r="L6" s="13">
         <f>IF(A6="","",DAYS(TODAY(),J6))</f>
         <v/>
       </c>
-      <c r="M6" s="11" t="n"/>
+      <c r="M6" s="11" t="inlineStr">
+        <is>
+          <t>Needs PHQ, $80 commission</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n"/>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Maurice Rondelez</t>
+        </is>
+      </c>
       <c r="B7" s="8" t="n"/>
       <c r="C7" s="8" t="n"/>
       <c r="D7" s="8" t="n"/>
       <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="9" t="n"/>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>200000</v>
+      </c>
       <c r="I7" s="9" t="n"/>
-      <c r="J7" s="8" t="n"/>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K7" s="8" t="n"/>
       <c r="L7" s="10">
         <f>IF(A7="","",DAYS(TODAY(),J7))</f>
@@ -1661,16 +1721,38 @@
       <c r="M7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n"/>
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Maurice Rondelez</t>
+        </is>
+      </c>
       <c r="B8" s="11" t="n"/>
       <c r="C8" s="11" t="n"/>
       <c r="D8" s="11" t="n"/>
-      <c r="E8" s="11" t="n"/>
-      <c r="F8" s="11" t="n"/>
-      <c r="G8" s="11" t="n"/>
-      <c r="H8" s="12" t="n"/>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="n">
+        <v>200000</v>
+      </c>
       <c r="I8" s="12" t="n"/>
-      <c r="J8" s="11" t="n"/>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K8" s="11" t="n"/>
       <c r="L8" s="13">
         <f>IF(A8="","",DAYS(TODAY(),J8))</f>
@@ -1679,16 +1761,30 @@
       <c r="M8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="n"/>
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Ruth Gilbert</t>
+        </is>
+      </c>
       <c r="B9" s="8" t="n"/>
       <c r="C9" s="8" t="n"/>
       <c r="D9" s="8" t="n"/>
       <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
       <c r="G9" s="8" t="n"/>
       <c r="H9" s="9" t="n"/>
-      <c r="I9" s="9" t="n"/>
-      <c r="J9" s="8" t="n"/>
+      <c r="I9" s="9" t="n">
+        <v>150000</v>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K9" s="8" t="n"/>
       <c r="L9" s="10">
         <f>IF(A9="","",DAYS(TODAY(),J9))</f>
@@ -1697,16 +1793,30 @@
       <c r="M9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n"/>
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Ruth Gilbert</t>
+        </is>
+      </c>
       <c r="B10" s="11" t="n"/>
       <c r="C10" s="11" t="n"/>
       <c r="D10" s="11" t="n"/>
       <c r="E10" s="11" t="n"/>
-      <c r="F10" s="11" t="n"/>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
       <c r="G10" s="11" t="n"/>
-      <c r="H10" s="12" t="n"/>
+      <c r="H10" s="12" t="n">
+        <v>150000</v>
+      </c>
       <c r="I10" s="12" t="n"/>
-      <c r="J10" s="11" t="n"/>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K10" s="11" t="n"/>
       <c r="L10" s="13">
         <f>IF(A10="","",DAYS(TODAY(),J10))</f>
@@ -1715,16 +1825,32 @@
       <c r="M10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="n"/>
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Jenn</t>
+        </is>
+      </c>
       <c r="B11" s="8" t="n"/>
       <c r="C11" s="8" t="n"/>
       <c r="D11" s="8" t="n"/>
       <c r="E11" s="8" t="n"/>
-      <c r="F11" s="8" t="n"/>
-      <c r="G11" s="8" t="n"/>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Life Insurance + Wealth</t>
+        </is>
+      </c>
       <c r="H11" s="9" t="n"/>
       <c r="I11" s="9" t="n"/>
-      <c r="J11" s="8" t="n"/>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K11" s="8" t="n"/>
       <c r="L11" s="10">
         <f>IF(A11="","",DAYS(TODAY(),J11))</f>
@@ -1733,16 +1859,32 @@
       <c r="M11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Nick</t>
+        </is>
+      </c>
       <c r="B12" s="11" t="n"/>
       <c r="C12" s="11" t="n"/>
       <c r="D12" s="11" t="n"/>
       <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>Life Insurance + Wealth</t>
+        </is>
+      </c>
       <c r="H12" s="12" t="n"/>
       <c r="I12" s="12" t="n"/>
-      <c r="J12" s="11" t="n"/>
+      <c r="J12" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K12" s="11" t="n"/>
       <c r="L12" s="13">
         <f>IF(A12="","",DAYS(TODAY(),J12))</f>
@@ -1751,16 +1893,32 @@
       <c r="M12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="n"/>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Jenn</t>
+        </is>
+      </c>
       <c r="B13" s="8" t="n"/>
       <c r="C13" s="8" t="n"/>
       <c r="D13" s="8" t="n"/>
       <c r="E13" s="8" t="n"/>
-      <c r="F13" s="8" t="n"/>
-      <c r="G13" s="8" t="n"/>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Life Insurance + Wealth</t>
+        </is>
+      </c>
       <c r="H13" s="9" t="n"/>
       <c r="I13" s="9" t="n"/>
-      <c r="J13" s="8" t="n"/>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K13" s="8" t="n"/>
       <c r="L13" s="10">
         <f>IF(A13="","",DAYS(TODAY(),J13))</f>
@@ -1769,16 +1927,32 @@
       <c r="M13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Nick</t>
+        </is>
+      </c>
       <c r="B14" s="11" t="n"/>
       <c r="C14" s="11" t="n"/>
       <c r="D14" s="11" t="n"/>
       <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>Life Insurance + Wealth</t>
+        </is>
+      </c>
       <c r="H14" s="12" t="n"/>
       <c r="I14" s="12" t="n"/>
-      <c r="J14" s="11" t="n"/>
+      <c r="J14" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K14" s="11" t="n"/>
       <c r="L14" s="13">
         <f>IF(A14="","",DAYS(TODAY(),J14))</f>
@@ -1787,17 +1961,43 @@
       <c r="M14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="n"/>
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Maurice Rondelez</t>
+        </is>
+      </c>
       <c r="B15" s="8" t="n"/>
       <c r="C15" s="8" t="n"/>
       <c r="D15" s="8" t="n"/>
-      <c r="E15" s="8" t="n"/>
-      <c r="F15" s="8" t="n"/>
-      <c r="G15" s="8" t="n"/>
-      <c r="H15" s="9" t="n"/>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="n">
+        <v>200000</v>
+      </c>
       <c r="I15" s="9" t="n"/>
-      <c r="J15" s="8" t="n"/>
-      <c r="K15" s="8" t="n"/>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
       <c r="L15" s="10">
         <f>IF(A15="","",DAYS(TODAY(),J15))</f>
         <v/>
@@ -1805,17 +2005,43 @@
       <c r="M15" s="8" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n"/>
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Maurice Rondelez</t>
+        </is>
+      </c>
       <c r="B16" s="11" t="n"/>
       <c r="C16" s="11" t="n"/>
       <c r="D16" s="11" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
-      <c r="H16" s="12" t="n"/>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="n">
+        <v>200000</v>
+      </c>
       <c r="I16" s="12" t="n"/>
-      <c r="J16" s="11" t="n"/>
-      <c r="K16" s="11" t="n"/>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="K16" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
       <c r="L16" s="13">
         <f>IF(A16="","",DAYS(TODAY(),J16))</f>
         <v/>
@@ -1823,34 +2049,86 @@
       <c r="M16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="n"/>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Maurice Rondelez</t>
+        </is>
+      </c>
       <c r="B17" s="8" t="n"/>
       <c r="C17" s="8" t="n"/>
-      <c r="D17" s="8" t="n"/>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="E17" s="8" t="n"/>
-      <c r="F17" s="8" t="n"/>
-      <c r="G17" s="8" t="n"/>
-      <c r="H17" s="9" t="n"/>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>200k</t>
+        </is>
+      </c>
       <c r="I17" s="9" t="n"/>
-      <c r="J17" s="8" t="n"/>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K17" s="8" t="n"/>
       <c r="L17" s="10">
         <f>IF(A17="","",DAYS(TODAY(),J17))</f>
         <v/>
       </c>
-      <c r="M17" s="8" t="n"/>
+      <c r="M17" s="8" t="inlineStr">
+        <is>
+          <t>elad</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n"/>
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Maurice Rondelez</t>
+        </is>
+      </c>
       <c r="B18" s="11" t="n"/>
       <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n"/>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Referral</t>
+        </is>
+      </c>
       <c r="E18" s="11" t="n"/>
-      <c r="F18" s="11" t="n"/>
-      <c r="G18" s="11" t="n"/>
-      <c r="H18" s="12" t="n"/>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>200k</t>
+        </is>
+      </c>
       <c r="I18" s="12" t="n"/>
-      <c r="J18" s="11" t="n"/>
+      <c r="J18" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K18" s="11" t="n"/>
       <c r="L18" s="13">
         <f>IF(A18="","",DAYS(TODAY(),J18))</f>
@@ -1859,17 +2137,43 @@
       <c r="M18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="n"/>
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Maurice Rondelez</t>
+        </is>
+      </c>
       <c r="B19" s="8" t="n"/>
       <c r="C19" s="8" t="n"/>
       <c r="D19" s="8" t="n"/>
-      <c r="E19" s="8" t="n"/>
-      <c r="F19" s="8" t="n"/>
-      <c r="G19" s="8" t="n"/>
-      <c r="H19" s="9" t="n"/>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="n">
+        <v>200000</v>
+      </c>
       <c r="I19" s="9" t="n"/>
-      <c r="J19" s="8" t="n"/>
-      <c r="K19" s="8" t="n"/>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="K19" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
       <c r="L19" s="10">
         <f>IF(A19="","",DAYS(TODAY(),J19))</f>
         <v/>
@@ -1877,17 +2181,43 @@
       <c r="M19" s="8" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n"/>
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Maurice Rondelez</t>
+        </is>
+      </c>
       <c r="B20" s="11" t="n"/>
       <c r="C20" s="11" t="n"/>
       <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="11" t="n"/>
-      <c r="G20" s="11" t="n"/>
-      <c r="H20" s="12" t="n"/>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="H20" s="12" t="n">
+        <v>200000</v>
+      </c>
       <c r="I20" s="12" t="n"/>
-      <c r="J20" s="11" t="n"/>
-      <c r="K20" s="11" t="n"/>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
       <c r="L20" s="13">
         <f>IF(A20="","",DAYS(TODAY(),J20))</f>
         <v/>
@@ -1895,16 +2225,28 @@
       <c r="M20" s="11" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="n"/>
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Office Manager</t>
+        </is>
+      </c>
       <c r="B21" s="8" t="n"/>
       <c r="C21" s="8" t="n"/>
       <c r="D21" s="8" t="n"/>
       <c r="E21" s="8" t="n"/>
-      <c r="F21" s="8" t="n"/>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
       <c r="G21" s="8" t="n"/>
       <c r="H21" s="9" t="n"/>
       <c r="I21" s="9" t="n"/>
-      <c r="J21" s="8" t="n"/>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K21" s="8" t="n"/>
       <c r="L21" s="10">
         <f>IF(A21="","",DAYS(TODAY(),J21))</f>
@@ -1913,58 +2255,132 @@
       <c r="M21" s="8" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="n"/>
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Kayla Cruz</t>
+        </is>
+      </c>
       <c r="B22" s="11" t="n"/>
       <c r="C22" s="11" t="n"/>
       <c r="D22" s="11" t="n"/>
       <c r="E22" s="11" t="n"/>
-      <c r="F22" s="11" t="n"/>
-      <c r="G22" s="11" t="n"/>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>Disability Insurance</t>
+        </is>
+      </c>
       <c r="H22" s="12" t="n"/>
-      <c r="I22" s="12" t="n"/>
-      <c r="J22" s="11" t="n"/>
+      <c r="I22" s="12" t="n">
+        <v>45000</v>
+      </c>
+      <c r="J22" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K22" s="11" t="n"/>
       <c r="L22" s="13">
         <f>IF(A22="","",DAYS(TODAY(),J22))</f>
         <v/>
       </c>
-      <c r="M22" s="11" t="n"/>
+      <c r="M22" s="11" t="inlineStr">
+        <is>
+          <t>DOB: Dec 24, 1990 | Admin Assistant at Premier | EI: Yes, Employer coverage: Yes (Premier) | WSIB: No | No injury history</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="n"/>
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Kayla Cruz</t>
+        </is>
+      </c>
       <c r="B23" s="8" t="n"/>
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="8" t="n"/>
-      <c r="E23" s="8" t="n"/>
-      <c r="F23" s="8" t="n"/>
-      <c r="G23" s="8" t="n"/>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Disability Insurance</t>
+        </is>
+      </c>
       <c r="H23" s="9" t="n"/>
-      <c r="I23" s="9" t="n"/>
-      <c r="J23" s="8" t="n"/>
+      <c r="I23" s="9" t="n">
+        <v>45000</v>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K23" s="8" t="n"/>
       <c r="L23" s="10">
         <f>IF(A23="","",DAYS(TODAY(),J23))</f>
         <v/>
       </c>
-      <c r="M23" s="8" t="n"/>
+      <c r="M23" s="8" t="inlineStr">
+        <is>
+          <t>DOB: Dec 24, 1990 | Admin Assistant | WSIB: No | EI: Yes | Net income: $45k | No injuries</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="n"/>
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Kayla Cruz</t>
+        </is>
+      </c>
       <c r="B24" s="11" t="n"/>
       <c r="C24" s="11" t="n"/>
       <c r="D24" s="11" t="n"/>
-      <c r="E24" s="11" t="n"/>
-      <c r="F24" s="11" t="n"/>
-      <c r="G24" s="11" t="n"/>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>Disability Insurance</t>
+        </is>
+      </c>
       <c r="H24" s="12" t="n"/>
-      <c r="I24" s="12" t="n"/>
-      <c r="J24" s="11" t="n"/>
+      <c r="I24" s="12" t="n">
+        <v>45000</v>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
       <c r="K24" s="11" t="n"/>
       <c r="L24" s="13">
         <f>IF(A24="","",DAYS(TODAY(),J24))</f>
         <v/>
       </c>
-      <c r="M24" s="11" t="n"/>
+      <c r="M24" s="11" t="inlineStr">
+        <is>
+          <t>Office worker, non-occupation disability quote. Female, age 45. Salary $45k.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n"/>

</xml_diff>